<commit_message>
descarte por restricición de vecindad
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isnelia.diaz\Documents\Coordinación de Extensión 2\Oferta Educación precedente\1. GECELCA\Grupos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FE619C-1BBF-438E-9610-21D74224EB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F5D2C8-6DF9-4556-A98E-E83C72C23806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -1271,7 +1271,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1418,273 +1418,6 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1692,6 +1425,277 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -2185,43 +2189,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H62"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.140625" customWidth="1"/>
-    <col min="2" max="2" width="41.42578125" style="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" style="47" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="17" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" customWidth="1"/>
+    <col min="2" max="2" width="41.44140625" style="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" style="47" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5546875" style="17" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" customWidth="1"/>
     <col min="7" max="7" width="42" style="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="106" t="s">
+    <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="108"/>
-    </row>
-    <row r="2" spans="1:8" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="105" t="s">
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="56"/>
+    </row>
+    <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="105"/>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="105"/>
-      <c r="H2" s="105"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -2247,1329 +2251,1329 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="44">
         <v>1</v>
       </c>
-      <c r="B4" s="139" t="s">
+      <c r="B4" s="50" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="139" t="s">
+      <c r="C4" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="140" t="s">
+      <c r="D4" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="E4" s="139" t="s">
+      <c r="E4" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="F4" s="140" t="s">
+      <c r="F4" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="G4" s="139" t="s">
+      <c r="G4" s="50" t="s">
         <v>95</v>
       </c>
-      <c r="H4" s="139" t="s">
+      <c r="H4" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="44">
         <f t="shared" ref="A5:A62" si="0">1+A4</f>
         <v>2</v>
       </c>
-      <c r="B5" s="139" t="s">
+      <c r="B5" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="C5" s="139" t="s">
+      <c r="C5" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="140" t="s">
+      <c r="D5" s="51" t="s">
         <v>149</v>
       </c>
-      <c r="E5" s="139" t="s">
+      <c r="E5" s="50" t="s">
         <v>150</v>
       </c>
-      <c r="F5" s="140" t="s">
+      <c r="F5" s="51" t="s">
         <v>151</v>
       </c>
-      <c r="G5" s="139" t="s">
+      <c r="G5" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="H5" s="139" t="s">
+      <c r="H5" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="44">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B6" s="139" t="s">
+      <c r="B6" s="50" t="s">
         <v>203</v>
       </c>
-      <c r="C6" s="139" t="s">
+      <c r="C6" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="140" t="s">
+      <c r="D6" s="51" t="s">
         <v>204</v>
       </c>
-      <c r="E6" s="139" t="s">
+      <c r="E6" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="140" t="s">
+      <c r="F6" s="51" t="s">
         <v>205</v>
       </c>
-      <c r="G6" s="139" t="s">
+      <c r="G6" s="50" t="s">
         <v>206</v>
       </c>
-      <c r="H6" s="139" t="s">
+      <c r="H6" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="44">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B7" s="139" t="s">
+      <c r="B7" s="50" t="s">
         <v>153</v>
       </c>
-      <c r="C7" s="139" t="s">
+      <c r="C7" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="140" t="s">
+      <c r="D7" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="E7" s="139" t="s">
+      <c r="E7" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="F7" s="140" t="s">
+      <c r="F7" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="G7" s="139" t="s">
+      <c r="G7" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="H7" s="139" t="s">
+      <c r="H7" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B8" s="139" t="s">
+      <c r="B8" s="50" t="s">
         <v>195</v>
       </c>
-      <c r="C8" s="139" t="s">
+      <c r="C8" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="140" t="s">
+      <c r="D8" s="51" t="s">
         <v>196</v>
       </c>
-      <c r="E8" s="139" t="s">
+      <c r="E8" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="F8" s="140" t="s">
+      <c r="F8" s="51" t="s">
         <v>197</v>
       </c>
-      <c r="G8" s="139" t="s">
+      <c r="G8" s="50" t="s">
         <v>198</v>
       </c>
-      <c r="H8" s="139" t="s">
+      <c r="H8" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="44">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B9" s="139" t="s">
+      <c r="B9" s="50" t="s">
         <v>176</v>
       </c>
-      <c r="C9" s="139" t="s">
+      <c r="C9" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="140" t="s">
+      <c r="D9" s="51" t="s">
         <v>177</v>
       </c>
-      <c r="E9" s="139" t="s">
+      <c r="E9" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="F9" s="140" t="s">
+      <c r="F9" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="G9" s="139" t="s">
+      <c r="G9" s="50" t="s">
         <v>180</v>
       </c>
-      <c r="H9" s="139" t="s">
+      <c r="H9" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="44">
+    <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="142">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B10" s="139" t="s">
+      <c r="B10" s="143" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="139" t="s">
+      <c r="C10" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="140" t="s">
+      <c r="D10" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="139" t="s">
+      <c r="E10" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="140" t="s">
+      <c r="F10" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="G10" s="139" t="s">
+      <c r="G10" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="139" t="s">
+      <c r="H10" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="44">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B11" s="139" t="s">
+      <c r="B11" s="143" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="139" t="s">
+      <c r="C11" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="140" t="s">
+      <c r="D11" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="E11" s="139" t="s">
+      <c r="E11" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="F11" s="140" t="s">
+      <c r="F11" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="G11" s="139" t="s">
+      <c r="G11" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="H11" s="139" t="s">
+      <c r="H11" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="44">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B12" s="139" t="s">
+      <c r="B12" s="143" t="s">
         <v>236</v>
       </c>
-      <c r="C12" s="139" t="s">
+      <c r="C12" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="140" t="s">
+      <c r="D12" s="51" t="s">
         <v>237</v>
       </c>
-      <c r="E12" s="139" t="s">
+      <c r="E12" s="50" t="s">
         <v>238</v>
       </c>
-      <c r="F12" s="140" t="s">
+      <c r="F12" s="51" t="s">
         <v>239</v>
       </c>
-      <c r="G12" s="139" t="s">
+      <c r="G12" s="50" t="s">
         <v>240</v>
       </c>
-      <c r="H12" s="139" t="s">
+      <c r="H12" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="44">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B13" s="139" t="s">
+      <c r="B13" s="143" t="s">
         <v>186</v>
       </c>
-      <c r="C13" s="139" t="s">
+      <c r="C13" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="140" t="s">
+      <c r="D13" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="E13" s="139" t="s">
+      <c r="E13" s="50" t="s">
         <v>183</v>
       </c>
-      <c r="F13" s="140" t="s">
+      <c r="F13" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="G13" s="139" t="s">
+      <c r="G13" s="50" t="s">
         <v>189</v>
       </c>
-      <c r="H13" s="139" t="s">
+      <c r="H13" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="44">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B14" s="139" t="s">
+      <c r="B14" s="143" t="s">
         <v>138</v>
       </c>
-      <c r="C14" s="139" t="s">
+      <c r="C14" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="140" t="s">
+      <c r="D14" s="51" t="s">
         <v>139</v>
       </c>
-      <c r="E14" s="139" t="s">
+      <c r="E14" s="50" t="s">
         <v>140</v>
       </c>
-      <c r="F14" s="140" t="s">
+      <c r="F14" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="G14" s="139" t="s">
+      <c r="G14" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="H14" s="139" t="s">
+      <c r="H14" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="44">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B15" s="139" t="s">
+      <c r="B15" s="143" t="s">
         <v>100</v>
       </c>
-      <c r="C15" s="139" t="s">
+      <c r="C15" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="140" t="s">
+      <c r="D15" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="E15" s="139" t="s">
+      <c r="E15" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="F15" s="140" t="s">
+      <c r="F15" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="G15" s="139" t="s">
+      <c r="G15" s="50" t="s">
         <v>104</v>
       </c>
-      <c r="H15" s="139" t="s">
+      <c r="H15" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="44">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B16" s="139" t="s">
+      <c r="B16" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="139" t="s">
+      <c r="C16" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="140" t="s">
+      <c r="D16" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="139" t="s">
+      <c r="E16" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="F16" s="140" t="s">
+      <c r="F16" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="G16" s="139" t="s">
+      <c r="G16" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="H16" s="139" t="s">
+      <c r="H16" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="44">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B17" s="139" t="s">
+      <c r="B17" s="50" t="s">
         <v>219</v>
       </c>
-      <c r="C17" s="139" t="s">
+      <c r="C17" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="140" t="s">
+      <c r="D17" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="E17" s="139" t="s">
+      <c r="E17" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F17" s="140" t="s">
+      <c r="F17" s="51" t="s">
         <v>221</v>
       </c>
-      <c r="G17" s="139" t="s">
+      <c r="G17" s="50" t="s">
         <v>222</v>
       </c>
-      <c r="H17" s="139" t="s">
+      <c r="H17" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="44">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B18" s="139" t="s">
+      <c r="B18" s="50" t="s">
         <v>251</v>
       </c>
-      <c r="C18" s="139" t="s">
+      <c r="C18" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="140" t="s">
+      <c r="D18" s="51" t="s">
         <v>252</v>
       </c>
-      <c r="E18" s="139" t="s">
+      <c r="E18" s="50" t="s">
         <v>248</v>
       </c>
-      <c r="F18" s="140" t="s">
+      <c r="F18" s="51" t="s">
         <v>253</v>
       </c>
-      <c r="G18" s="139" t="s">
+      <c r="G18" s="50" t="s">
         <v>254</v>
       </c>
-      <c r="H18" s="139" t="s">
+      <c r="H18" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="44">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B19" s="139" t="s">
+      <c r="B19" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="139" t="s">
+      <c r="C19" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="140" t="s">
+      <c r="D19" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="E19" s="139" t="s">
+      <c r="E19" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F19" s="140" t="s">
+      <c r="F19" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="G19" s="139" t="s">
+      <c r="G19" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="H19" s="139" t="s">
+      <c r="H19" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="44">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B20" s="139" t="s">
+      <c r="B20" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="139" t="s">
+      <c r="C20" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="140" t="s">
+      <c r="D20" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="E20" s="139" t="s">
+      <c r="E20" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F20" s="140" t="s">
+      <c r="F20" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="139" t="s">
+      <c r="G20" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="H20" s="139" t="s">
+      <c r="H20" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="44">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B21" s="139" t="s">
+      <c r="B21" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="C21" s="139" t="s">
+      <c r="C21" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="141" t="s">
+      <c r="D21" s="52" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="139" t="s">
+      <c r="E21" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="F21" s="140" t="s">
+      <c r="F21" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="G21" s="139" t="s">
+      <c r="G21" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="H21" s="139" t="s">
+      <c r="H21" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="44">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B22" s="139" t="s">
+      <c r="B22" s="50" t="s">
         <v>124</v>
       </c>
-      <c r="C22" s="139" t="s">
+      <c r="C22" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="140" t="s">
+      <c r="D22" s="51" t="s">
         <v>125</v>
       </c>
-      <c r="E22" s="139" t="s">
+      <c r="E22" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="F22" s="140" t="s">
+      <c r="F22" s="51" t="s">
         <v>127</v>
       </c>
-      <c r="G22" s="139" t="s">
+      <c r="G22" s="50" t="s">
         <v>128</v>
       </c>
-      <c r="H22" s="139" t="s">
+      <c r="H22" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="44">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B23" s="139" t="s">
+      <c r="B23" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="C23" s="139" t="s">
+      <c r="C23" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="140" t="s">
+      <c r="D23" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="E23" s="139" t="s">
+      <c r="E23" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="F23" s="140" t="s">
+      <c r="F23" s="51" t="s">
         <v>170</v>
       </c>
-      <c r="G23" s="139" t="s">
+      <c r="G23" s="50" t="s">
         <v>171</v>
       </c>
-      <c r="H23" s="139" t="s">
+      <c r="H23" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="44">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B24" s="139" t="s">
+      <c r="B24" s="50" t="s">
         <v>199</v>
       </c>
-      <c r="C24" s="139" t="s">
+      <c r="C24" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="140" t="s">
+      <c r="D24" s="51" t="s">
         <v>200</v>
       </c>
-      <c r="E24" s="139" t="s">
+      <c r="E24" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="140" t="s">
+      <c r="F24" s="51" t="s">
         <v>201</v>
       </c>
-      <c r="G24" s="139" t="s">
+      <c r="G24" s="50" t="s">
         <v>202</v>
       </c>
-      <c r="H24" s="139" t="s">
+      <c r="H24" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="44">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B25" s="139" t="s">
+      <c r="B25" s="50" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="139" t="s">
+      <c r="C25" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="140" t="s">
+      <c r="D25" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="139" t="s">
+      <c r="E25" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F25" s="140" t="s">
+      <c r="F25" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="G25" s="139" t="s">
+      <c r="G25" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="H25" s="139" t="s">
+      <c r="H25" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="44">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="B26" s="139" t="s">
+      <c r="B26" s="50" t="s">
         <v>241</v>
       </c>
-      <c r="C26" s="139" t="s">
+      <c r="C26" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="140" t="s">
+      <c r="D26" s="51" t="s">
         <v>242</v>
       </c>
-      <c r="E26" s="139" t="s">
+      <c r="E26" s="50" t="s">
         <v>243</v>
       </c>
-      <c r="F26" s="140" t="s">
+      <c r="F26" s="51" t="s">
         <v>244</v>
       </c>
-      <c r="G26" s="139" t="s">
+      <c r="G26" s="50" t="s">
         <v>245</v>
       </c>
-      <c r="H26" s="139" t="s">
+      <c r="H26" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="44">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="B27" s="139" t="s">
+      <c r="B27" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="139" t="s">
+      <c r="C27" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="140" t="s">
+      <c r="D27" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="139" t="s">
+      <c r="E27" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F27" s="141" t="s">
+      <c r="F27" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="G27" s="139" t="s">
+      <c r="G27" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="H27" s="139" t="s">
+      <c r="H27" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="44">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="B28" s="139" t="s">
+      <c r="B28" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="139" t="s">
+      <c r="C28" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="140" t="s">
+      <c r="D28" s="51" t="s">
         <v>78</v>
       </c>
-      <c r="E28" s="139" t="s">
+      <c r="E28" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="F28" s="140" t="s">
+      <c r="F28" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="139" t="s">
+      <c r="G28" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="H28" s="139" t="s">
+      <c r="H28" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="44">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B29" s="139" t="s">
+      <c r="B29" s="50" t="s">
         <v>246</v>
       </c>
-      <c r="C29" s="139" t="s">
+      <c r="C29" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="140" t="s">
+      <c r="D29" s="51" t="s">
         <v>247</v>
       </c>
-      <c r="E29" s="139" t="s">
+      <c r="E29" s="50" t="s">
         <v>248</v>
       </c>
-      <c r="F29" s="140" t="s">
+      <c r="F29" s="51" t="s">
         <v>249</v>
       </c>
-      <c r="G29" s="139" t="s">
+      <c r="G29" s="50" t="s">
         <v>250</v>
       </c>
-      <c r="H29" s="139" t="s">
+      <c r="H29" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="44">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="B30" s="139" t="s">
+      <c r="B30" s="50" t="s">
         <v>223</v>
       </c>
-      <c r="C30" s="139" t="s">
+      <c r="C30" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="140" t="s">
+      <c r="D30" s="51" t="s">
         <v>224</v>
       </c>
-      <c r="E30" s="139" t="s">
+      <c r="E30" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F30" s="140" t="s">
+      <c r="F30" s="51" t="s">
         <v>225</v>
       </c>
-      <c r="G30" s="139" t="s">
+      <c r="G30" s="50" t="s">
         <v>226</v>
       </c>
-      <c r="H30" s="139" t="s">
+      <c r="H30" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="44">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B31" s="139" t="s">
+      <c r="B31" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="C31" s="139" t="s">
+      <c r="C31" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="140" t="s">
+      <c r="D31" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="E31" s="139" t="s">
+      <c r="E31" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F31" s="140" t="s">
+      <c r="F31" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="G31" s="139" t="s">
+      <c r="G31" s="50" t="s">
         <v>210</v>
       </c>
-      <c r="H31" s="139" t="s">
+      <c r="H31" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="44">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="B32" s="139" t="s">
+      <c r="B32" s="50" t="s">
         <v>211</v>
       </c>
-      <c r="C32" s="139" t="s">
+      <c r="C32" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="140" t="s">
+      <c r="D32" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="E32" s="139" t="s">
+      <c r="E32" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="140" t="s">
+      <c r="F32" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="G32" s="139" t="s">
+      <c r="G32" s="50" t="s">
         <v>214</v>
       </c>
-      <c r="H32" s="139" t="s">
+      <c r="H32" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="44">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B33" s="139" t="s">
+      <c r="B33" s="50" t="s">
         <v>215</v>
       </c>
-      <c r="C33" s="139" t="s">
+      <c r="C33" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="140" t="s">
+      <c r="D33" s="51" t="s">
         <v>216</v>
       </c>
-      <c r="E33" s="139" t="s">
+      <c r="E33" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F33" s="140" t="s">
+      <c r="F33" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="G33" s="139" t="s">
+      <c r="G33" s="50" t="s">
         <v>218</v>
       </c>
-      <c r="H33" s="139" t="s">
+      <c r="H33" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="44">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="B34" s="139" t="s">
+      <c r="B34" s="50" t="s">
         <v>227</v>
       </c>
-      <c r="C34" s="139" t="s">
+      <c r="C34" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D34" s="140" t="s">
+      <c r="D34" s="51" t="s">
         <v>228</v>
       </c>
-      <c r="E34" s="139" t="s">
+      <c r="E34" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F34" s="140" t="s">
+      <c r="F34" s="51" t="s">
         <v>229</v>
       </c>
-      <c r="G34" s="139" t="s">
+      <c r="G34" s="50" t="s">
         <v>230</v>
       </c>
-      <c r="H34" s="139" t="s">
+      <c r="H34" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="44">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B35" s="139" t="s">
+      <c r="B35" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="C35" s="139" t="s">
+      <c r="C35" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="140" t="s">
+      <c r="D35" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="E35" s="139" t="s">
+      <c r="E35" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="F35" s="140" t="s">
+      <c r="F35" s="51" t="s">
         <v>75</v>
       </c>
-      <c r="G35" s="139" t="s">
+      <c r="G35" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H35" s="139" t="s">
+      <c r="H35" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="44">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="B36" s="139" t="s">
+      <c r="B36" s="50" t="s">
         <v>129</v>
       </c>
-      <c r="C36" s="139" t="s">
+      <c r="C36" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D36" s="140" t="s">
+      <c r="D36" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="139" t="s">
+      <c r="E36" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="F36" s="140" t="s">
+      <c r="F36" s="51" t="s">
         <v>132</v>
       </c>
-      <c r="G36" s="139" t="s">
+      <c r="G36" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="H36" s="139" t="s">
+      <c r="H36" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="44">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="B37" s="139" t="s">
+      <c r="B37" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="C37" s="139" t="s">
+      <c r="C37" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D37" s="140" t="s">
+      <c r="D37" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="E37" s="139" t="s">
+      <c r="E37" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="F37" s="140" t="s">
+      <c r="F37" s="51" t="s">
         <v>84</v>
       </c>
-      <c r="G37" s="139" t="s">
+      <c r="G37" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="H37" s="139" t="s">
+      <c r="H37" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="44">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="B38" s="139" t="s">
+      <c r="B38" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="139" t="s">
+      <c r="C38" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="140" t="s">
+      <c r="D38" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="E38" s="139" t="s">
+      <c r="E38" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F38" s="140" t="s">
+      <c r="F38" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="G38" s="139" t="s">
+      <c r="G38" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="H38" s="139" t="s">
+      <c r="H38" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="44">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="B39" s="139" t="s">
+      <c r="B39" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="C39" s="139" t="s">
+      <c r="C39" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D39" s="140" t="s">
+      <c r="D39" s="51" t="s">
         <v>61</v>
       </c>
-      <c r="E39" s="139" t="s">
+      <c r="E39" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F39" s="140" t="s">
+      <c r="F39" s="51" t="s">
         <v>62</v>
       </c>
-      <c r="G39" s="139" t="s">
+      <c r="G39" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="H39" s="139" t="s">
+      <c r="H39" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="44">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="B40" s="139" t="s">
+      <c r="B40" s="50" t="s">
         <v>181</v>
       </c>
-      <c r="C40" s="139" t="s">
+      <c r="C40" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D40" s="140" t="s">
+      <c r="D40" s="51" t="s">
         <v>182</v>
       </c>
-      <c r="E40" s="139" t="s">
+      <c r="E40" s="50" t="s">
         <v>183</v>
       </c>
-      <c r="F40" s="140" t="s">
+      <c r="F40" s="51" t="s">
         <v>184</v>
       </c>
-      <c r="G40" s="139" t="s">
+      <c r="G40" s="50" t="s">
         <v>185</v>
       </c>
-      <c r="H40" s="139" t="s">
+      <c r="H40" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="44">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="B41" s="139" t="s">
+      <c r="B41" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="C41" s="139" t="s">
+      <c r="C41" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D41" s="140" t="s">
+      <c r="D41" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="E41" s="139" t="s">
+      <c r="E41" s="50" t="s">
         <v>52</v>
       </c>
-      <c r="F41" s="140" t="s">
+      <c r="F41" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="G41" s="139" t="s">
+      <c r="G41" s="50" t="s">
         <v>54</v>
       </c>
-      <c r="H41" s="139" t="s">
+      <c r="H41" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="44">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="B42" s="139" t="s">
+      <c r="B42" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="C42" s="139" t="s">
+      <c r="C42" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D42" s="140" t="s">
+      <c r="D42" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="E42" s="139" t="s">
+      <c r="E42" s="50" t="s">
         <v>145</v>
       </c>
-      <c r="F42" s="140" t="s">
+      <c r="F42" s="51" t="s">
         <v>146</v>
       </c>
-      <c r="G42" s="139" t="s">
+      <c r="G42" s="50" t="s">
         <v>147</v>
       </c>
-      <c r="H42" s="139" t="s">
+      <c r="H42" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="44">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="B43" s="139" t="s">
+      <c r="B43" s="50" t="s">
         <v>172</v>
       </c>
-      <c r="C43" s="139" t="s">
+      <c r="C43" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D43" s="140" t="s">
+      <c r="D43" s="51" t="s">
         <v>173</v>
       </c>
-      <c r="E43" s="139" t="s">
+      <c r="E43" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="F43" s="140" t="s">
+      <c r="F43" s="51" t="s">
         <v>174</v>
       </c>
-      <c r="G43" s="139" t="s">
+      <c r="G43" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="H43" s="139" t="s">
+      <c r="H43" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="44">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="B44" s="139" t="s">
+      <c r="B44" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="C44" s="139" t="s">
+      <c r="C44" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D44" s="140" t="s">
+      <c r="D44" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="E44" s="139" t="s">
+      <c r="E44" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="F44" s="140" t="s">
+      <c r="F44" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="G44" s="139" t="s">
+      <c r="G44" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="H44" s="139" t="s">
+      <c r="H44" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="44">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="B45" s="139" t="s">
+      <c r="B45" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="C45" s="139" t="s">
+      <c r="C45" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D45" s="140" t="s">
+      <c r="D45" s="51" t="s">
         <v>120</v>
       </c>
-      <c r="E45" s="139" t="s">
+      <c r="E45" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="F45" s="140" t="s">
+      <c r="F45" s="51" t="s">
         <v>122</v>
       </c>
-      <c r="G45" s="139" t="s">
+      <c r="G45" s="50" t="s">
         <v>123</v>
       </c>
-      <c r="H45" s="139" t="s">
+      <c r="H45" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="44">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="B46" s="139" t="s">
+      <c r="B46" s="50" t="s">
         <v>96</v>
       </c>
-      <c r="C46" s="139" t="s">
+      <c r="C46" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D46" s="140" t="s">
+      <c r="D46" s="51" t="s">
         <v>97</v>
       </c>
-      <c r="E46" s="139" t="s">
+      <c r="E46" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="F46" s="140" t="s">
+      <c r="F46" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="G46" s="139" t="s">
+      <c r="G46" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="H46" s="139" t="s">
+      <c r="H46" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="44">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="B47" s="139" t="s">
+      <c r="B47" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="C47" s="139" t="s">
+      <c r="C47" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D47" s="140" t="s">
+      <c r="D47" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="E47" s="139" t="s">
+      <c r="E47" s="50" t="s">
         <v>164</v>
       </c>
-      <c r="F47" s="140" t="s">
+      <c r="F47" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="G47" s="139" t="s">
+      <c r="G47" s="50" t="s">
         <v>166</v>
       </c>
-      <c r="H47" s="139" t="s">
+      <c r="H47" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="44">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="B48" s="139" t="s">
+      <c r="B48" s="50" t="s">
         <v>134</v>
       </c>
-      <c r="C48" s="139" t="s">
+      <c r="C48" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="140" t="s">
+      <c r="D48" s="51" t="s">
         <v>135</v>
       </c>
-      <c r="E48" s="139" t="s">
+      <c r="E48" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="F48" s="140" t="s">
+      <c r="F48" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="G48" s="139" t="s">
+      <c r="G48" s="50" t="s">
         <v>137</v>
       </c>
-      <c r="H48" s="139" t="s">
+      <c r="H48" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="44">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="B49" s="139" t="s">
+      <c r="B49" s="50" t="s">
         <v>105</v>
       </c>
-      <c r="C49" s="139" t="s">
+      <c r="C49" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D49" s="140" t="s">
+      <c r="D49" s="51" t="s">
         <v>106</v>
       </c>
-      <c r="E49" s="139" t="s">
+      <c r="E49" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="F49" s="140" t="s">
+      <c r="F49" s="51" t="s">
         <v>107</v>
       </c>
-      <c r="G49" s="139" t="s">
+      <c r="G49" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="H49" s="139" t="s">
+      <c r="H49" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="44">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="B50" s="139" t="s">
+      <c r="B50" s="50" t="s">
         <v>231</v>
       </c>
-      <c r="C50" s="139" t="s">
+      <c r="C50" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D50" s="140" t="s">
+      <c r="D50" s="51" t="s">
         <v>232</v>
       </c>
-      <c r="E50" s="139" t="s">
+      <c r="E50" s="50" t="s">
         <v>233</v>
       </c>
-      <c r="F50" s="140" t="s">
+      <c r="F50" s="51" t="s">
         <v>234</v>
       </c>
-      <c r="G50" s="139" t="s">
+      <c r="G50" s="50" t="s">
         <v>235</v>
       </c>
-      <c r="H50" s="139" t="s">
+      <c r="H50" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="44">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="B51" s="139" t="s">
+      <c r="B51" s="50" t="s">
         <v>190</v>
       </c>
-      <c r="C51" s="139" t="s">
+      <c r="C51" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D51" s="140" t="s">
+      <c r="D51" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="E51" s="139" t="s">
+      <c r="E51" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="F51" s="140" t="s">
+      <c r="F51" s="51" t="s">
         <v>193</v>
       </c>
-      <c r="G51" s="139" t="s">
+      <c r="G51" s="50" t="s">
         <v>194</v>
       </c>
-      <c r="H51" s="139" t="s">
+      <c r="H51" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="44">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="B52" s="139" t="s">
+      <c r="B52" s="50" t="s">
         <v>109</v>
       </c>
-      <c r="C52" s="139" t="s">
+      <c r="C52" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D52" s="140" t="s">
+      <c r="D52" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="E52" s="139" t="s">
+      <c r="E52" s="50" t="s">
         <v>111</v>
       </c>
-      <c r="F52" s="140" t="s">
+      <c r="F52" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="G52" s="139" t="s">
+      <c r="G52" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="H52" s="139" t="s">
+      <c r="H52" s="50" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="44">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -3582,7 +3586,7 @@
       <c r="G53" s="18"/>
       <c r="H53" s="49"/>
     </row>
-    <row r="54" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="44">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -3595,7 +3599,7 @@
       <c r="G54" s="18"/>
       <c r="H54" s="49"/>
     </row>
-    <row r="55" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="44">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -3608,7 +3612,7 @@
       <c r="G55" s="18"/>
       <c r="H55" s="49"/>
     </row>
-    <row r="56" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="44">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -3621,7 +3625,7 @@
       <c r="G56" s="18"/>
       <c r="H56" s="49"/>
     </row>
-    <row r="57" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="44">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -3634,7 +3638,7 @@
       <c r="G57" s="18"/>
       <c r="H57" s="49"/>
     </row>
-    <row r="58" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="44">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -3647,7 +3651,7 @@
       <c r="G58" s="18"/>
       <c r="H58" s="49"/>
     </row>
-    <row r="59" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="44">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -3660,7 +3664,7 @@
       <c r="G59" s="18"/>
       <c r="H59" s="49"/>
     </row>
-    <row r="60" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="44">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3673,7 +3677,7 @@
       <c r="G60" s="18"/>
       <c r="H60" s="49"/>
     </row>
-    <row r="61" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="44">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -3686,7 +3690,7 @@
       <c r="G61" s="18"/>
       <c r="H61" s="15"/>
     </row>
-    <row r="62" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="44">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -3713,187 +3717,187 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AE64"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="7" width="7.28515625" customWidth="1"/>
-    <col min="8" max="8" width="7.28515625" style="2" customWidth="1"/>
-    <col min="9" max="16" width="7.28515625" customWidth="1"/>
-    <col min="17" max="17" width="7.28515625" style="2" customWidth="1"/>
-    <col min="18" max="25" width="7.28515625" customWidth="1"/>
-    <col min="26" max="26" width="7.28515625" style="2" customWidth="1"/>
-    <col min="27" max="30" width="7.28515625" customWidth="1"/>
-    <col min="31" max="31" width="7.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="7" width="7.33203125" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" style="2" customWidth="1"/>
+    <col min="9" max="16" width="7.33203125" customWidth="1"/>
+    <col min="17" max="17" width="7.33203125" style="2" customWidth="1"/>
+    <col min="18" max="25" width="7.33203125" customWidth="1"/>
+    <col min="26" max="26" width="7.33203125" style="2" customWidth="1"/>
+    <col min="27" max="30" width="7.33203125" customWidth="1"/>
+    <col min="31" max="31" width="7.33203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="116" t="s">
+    <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
-      <c r="AD1" s="116"/>
-      <c r="AE1" s="116"/>
-    </row>
-    <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="78" t="s">
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="64"/>
+      <c r="O1" s="64"/>
+      <c r="P1" s="64"/>
+      <c r="Q1" s="64"/>
+      <c r="R1" s="64"/>
+      <c r="S1" s="64"/>
+      <c r="T1" s="64"/>
+      <c r="U1" s="64"/>
+      <c r="V1" s="64"/>
+      <c r="W1" s="64"/>
+      <c r="X1" s="64"/>
+      <c r="Y1" s="64"/>
+      <c r="Z1" s="64"/>
+      <c r="AA1" s="64"/>
+      <c r="AB1" s="64"/>
+      <c r="AC1" s="64"/>
+      <c r="AD1" s="64"/>
+      <c r="AE1" s="64"/>
+    </row>
+    <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="78" t="s">
+      <c r="C2" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="132" t="s">
+      <c r="D2" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="134"/>
-      <c r="I2" s="117" t="s">
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="118"/>
-      <c r="K2" s="118"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
-      <c r="N2" s="118"/>
-      <c r="O2" s="118"/>
-      <c r="P2" s="118"/>
-      <c r="Q2" s="119"/>
-      <c r="R2" s="126" t="s">
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="68"/>
+      <c r="P2" s="68"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="127"/>
-      <c r="T2" s="127"/>
-      <c r="U2" s="127"/>
-      <c r="V2" s="127"/>
-      <c r="W2" s="127"/>
-      <c r="X2" s="127"/>
-      <c r="Y2" s="127"/>
-      <c r="Z2" s="128"/>
-      <c r="AA2" s="109" t="s">
+      <c r="S2" s="77"/>
+      <c r="T2" s="77"/>
+      <c r="U2" s="77"/>
+      <c r="V2" s="77"/>
+      <c r="W2" s="77"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="77"/>
+      <c r="Z2" s="78"/>
+      <c r="AA2" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="110"/>
-      <c r="AC2" s="110"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="111"/>
-    </row>
-    <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="79"/>
-      <c r="B3" s="77"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="135" t="s">
+      <c r="AB2" s="58"/>
+      <c r="AC2" s="58"/>
+      <c r="AD2" s="58"/>
+      <c r="AE2" s="59"/>
+    </row>
+    <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="66"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="136"/>
-      <c r="F3" s="136"/>
-      <c r="G3" s="136"/>
-      <c r="H3" s="137"/>
-      <c r="I3" s="120" t="s">
+      <c r="E3" s="86"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="121"/>
-      <c r="K3" s="121"/>
-      <c r="L3" s="121"/>
-      <c r="M3" s="121"/>
-      <c r="N3" s="121"/>
-      <c r="O3" s="121"/>
-      <c r="P3" s="121"/>
-      <c r="Q3" s="122"/>
-      <c r="R3" s="129" t="s">
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71"/>
+      <c r="P3" s="71"/>
+      <c r="Q3" s="72"/>
+      <c r="R3" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="130"/>
-      <c r="T3" s="130"/>
-      <c r="U3" s="130"/>
-      <c r="V3" s="130"/>
-      <c r="W3" s="130"/>
-      <c r="X3" s="130"/>
-      <c r="Y3" s="130"/>
-      <c r="Z3" s="131"/>
-      <c r="AA3" s="112" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="113"/>
-      <c r="AC3" s="113"/>
-      <c r="AD3" s="113"/>
-      <c r="AE3" s="114"/>
-    </row>
-    <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="79"/>
-      <c r="B4" s="77"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="138" t="s">
+      <c r="S3" s="80"/>
+      <c r="T3" s="80"/>
+      <c r="U3" s="80"/>
+      <c r="V3" s="80"/>
+      <c r="W3" s="80"/>
+      <c r="X3" s="80"/>
+      <c r="Y3" s="80"/>
+      <c r="Z3" s="81"/>
+      <c r="AA3" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="61"/>
+      <c r="AC3" s="61"/>
+      <c r="AD3" s="61"/>
+      <c r="AE3" s="62"/>
+    </row>
+    <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="66"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="124"/>
-      <c r="F4" s="124"/>
-      <c r="G4" s="125"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="75"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="123" t="s">
+      <c r="I4" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="124"/>
-      <c r="K4" s="124"/>
-      <c r="L4" s="124"/>
-      <c r="M4" s="124"/>
-      <c r="N4" s="124"/>
-      <c r="O4" s="124"/>
-      <c r="P4" s="125"/>
+      <c r="J4" s="74"/>
+      <c r="K4" s="74"/>
+      <c r="L4" s="74"/>
+      <c r="M4" s="74"/>
+      <c r="N4" s="74"/>
+      <c r="O4" s="74"/>
+      <c r="P4" s="75"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="123" t="s">
+      <c r="R4" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="124"/>
-      <c r="T4" s="124"/>
-      <c r="U4" s="124"/>
-      <c r="V4" s="124"/>
-      <c r="W4" s="124"/>
-      <c r="X4" s="124"/>
-      <c r="Y4" s="125"/>
+      <c r="S4" s="74"/>
+      <c r="T4" s="74"/>
+      <c r="U4" s="74"/>
+      <c r="V4" s="74"/>
+      <c r="W4" s="74"/>
+      <c r="X4" s="74"/>
+      <c r="Y4" s="75"/>
       <c r="Z4" s="13"/>
-      <c r="AA4" s="115" t="s">
+      <c r="AA4" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="AB4" s="115"/>
-      <c r="AC4" s="115"/>
-      <c r="AD4" s="115"/>
+      <c r="AB4" s="63"/>
+      <c r="AC4" s="63"/>
+      <c r="AD4" s="63"/>
       <c r="AE4" s="3"/>
     </row>
-    <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="79"/>
-      <c r="B5" s="77"/>
-      <c r="C5" s="79"/>
+    <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="66"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="66"/>
       <c r="D5" s="34"/>
       <c r="E5" s="34"/>
       <c r="F5" s="34"/>
@@ -3931,7 +3935,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>1</v>
       </c>
@@ -3984,7 +3988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>2</v>
       </c>
@@ -4037,7 +4041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A8" s="21">
         <v>3</v>
       </c>
@@ -4090,7 +4094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A9" s="21">
         <v>4</v>
       </c>
@@ -4143,7 +4147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A10" s="21">
         <v>5</v>
       </c>
@@ -4196,7 +4200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A11" s="21">
         <v>6</v>
       </c>
@@ -4249,7 +4253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A12" s="21">
         <v>7</v>
       </c>
@@ -4302,7 +4306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A13" s="21">
         <v>8</v>
       </c>
@@ -4355,7 +4359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A14" s="21">
         <v>9</v>
       </c>
@@ -4408,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A15" s="21">
         <v>10</v>
       </c>
@@ -4461,7 +4465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A16" s="21">
         <v>11</v>
       </c>
@@ -4514,7 +4518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A17" s="21">
         <v>12</v>
       </c>
@@ -4567,7 +4571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A18" s="21">
         <v>13</v>
       </c>
@@ -4620,7 +4624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A19" s="21">
         <v>14</v>
       </c>
@@ -4673,7 +4677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A20" s="21">
         <v>15</v>
       </c>
@@ -4726,7 +4730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A21" s="21">
         <v>16</v>
       </c>
@@ -4779,7 +4783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A22" s="21">
         <v>17</v>
       </c>
@@ -4832,7 +4836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A23" s="21">
         <v>18</v>
       </c>
@@ -4885,7 +4889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A24" s="21">
         <v>19</v>
       </c>
@@ -4938,7 +4942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A25" s="21">
         <v>20</v>
       </c>
@@ -4991,7 +4995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A26" s="21">
         <v>21</v>
       </c>
@@ -5044,7 +5048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A27" s="21">
         <v>22</v>
       </c>
@@ -5097,7 +5101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A28" s="21">
         <v>23</v>
       </c>
@@ -5150,7 +5154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A29" s="21">
         <v>24</v>
       </c>
@@ -5203,7 +5207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A30" s="21">
         <v>25</v>
       </c>
@@ -5256,7 +5260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A31" s="21">
         <v>26</v>
       </c>
@@ -5309,7 +5313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A32" s="21">
         <v>27</v>
       </c>
@@ -5362,7 +5366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A33" s="21">
         <v>28</v>
       </c>
@@ -5415,7 +5419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A34" s="21">
         <v>29</v>
       </c>
@@ -5468,7 +5472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A35" s="21">
         <v>30</v>
       </c>
@@ -5521,7 +5525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" s="20" customFormat="1" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A36" s="21">
         <v>31</v>
       </c>
@@ -5574,7 +5578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A37" s="21">
         <v>32</v>
       </c>
@@ -5627,7 +5631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A38" s="21">
         <v>33</v>
       </c>
@@ -5680,7 +5684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A39" s="21">
         <v>34</v>
       </c>
@@ -5733,7 +5737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A40" s="21">
         <v>35</v>
       </c>
@@ -5786,7 +5790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A41" s="21">
         <v>36</v>
       </c>
@@ -5839,7 +5843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A42" s="21">
         <v>37</v>
       </c>
@@ -5892,7 +5896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A43" s="21">
         <v>38</v>
       </c>
@@ -5945,7 +5949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A44" s="21">
         <v>39</v>
       </c>
@@ -5998,7 +6002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A45" s="21">
         <v>40</v>
       </c>
@@ -6051,7 +6055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A46" s="21">
         <v>41</v>
       </c>
@@ -6104,7 +6108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A47" s="21">
         <v>42</v>
       </c>
@@ -6157,7 +6161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A48" s="21">
         <v>43</v>
       </c>
@@ -6210,7 +6214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A49" s="21">
         <v>44</v>
       </c>
@@ -6263,7 +6267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A50" s="21">
         <v>45</v>
       </c>
@@ -6316,7 +6320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A51" s="21">
         <v>46</v>
       </c>
@@ -6369,7 +6373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A52" s="21">
         <v>47</v>
       </c>
@@ -6422,7 +6426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A53" s="21">
         <v>48</v>
       </c>
@@ -6475,7 +6479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A54" s="21">
         <v>49</v>
       </c>
@@ -6528,7 +6532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A55" s="21">
         <v>50</v>
       </c>
@@ -6581,7 +6585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A56" s="21">
         <v>51</v>
       </c>
@@ -6634,7 +6638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A57" s="21">
         <v>52</v>
       </c>
@@ -6687,7 +6691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A58" s="21">
         <v>53</v>
       </c>
@@ -6740,7 +6744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A59" s="21">
         <v>54</v>
       </c>
@@ -6793,7 +6797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A60" s="21">
         <v>55</v>
       </c>
@@ -6846,7 +6850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A61" s="21">
         <v>56</v>
       </c>
@@ -6899,7 +6903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A62" s="21">
         <v>57</v>
       </c>
@@ -6952,7 +6956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A63" s="21">
         <v>58</v>
       </c>
@@ -7005,7 +7009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:31" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A64" s="21">
         <v>59</v>
       </c>
@@ -7087,143 +7091,143 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:T74"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="34.5703125" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="7.28515625" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="34.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="7.33203125" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
-    <col min="10" max="10" width="5.7109375" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" style="2" customWidth="1"/>
-    <col min="12" max="15" width="6.7109375" customWidth="1"/>
-    <col min="16" max="16" width="8.28515625" style="2" customWidth="1"/>
-    <col min="17" max="19" width="7.7109375" customWidth="1"/>
-    <col min="20" max="20" width="7.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" customWidth="1"/>
+    <col min="11" max="11" width="8.5546875" style="2" customWidth="1"/>
+    <col min="12" max="15" width="6.6640625" customWidth="1"/>
+    <col min="16" max="16" width="8.33203125" style="2" customWidth="1"/>
+    <col min="17" max="19" width="7.6640625" customWidth="1"/>
+    <col min="20" max="20" width="7.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="80" t="s">
+    <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="91" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="80"/>
-      <c r="I1" s="80"/>
-      <c r="J1" s="80"/>
-      <c r="K1" s="80"/>
-      <c r="L1" s="80"/>
-      <c r="M1" s="80"/>
-      <c r="N1" s="80"/>
-      <c r="O1" s="80"/>
-      <c r="P1" s="80"/>
-      <c r="Q1" s="80"/>
-      <c r="R1" s="80"/>
-      <c r="S1" s="80"/>
-      <c r="T1" s="80"/>
-    </row>
-    <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="62" t="s">
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+    </row>
+    <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="128" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="78" t="s">
+      <c r="C2" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="50" t="str">
+      <c r="D2" s="119" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="51"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="50" t="str">
+      <c r="E2" s="120"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="119" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="52"/>
-      <c r="L2" s="50" t="s">
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="121"/>
+      <c r="L2" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="51"/>
-      <c r="N2" s="51"/>
-      <c r="O2" s="51"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="50" t="str">
+      <c r="M2" s="120"/>
+      <c r="N2" s="120"/>
+      <c r="O2" s="120"/>
+      <c r="P2" s="121"/>
+      <c r="Q2" s="119" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="51"/>
-      <c r="S2" s="51"/>
-      <c r="T2" s="52"/>
-    </row>
-    <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="63"/>
-      <c r="B3" s="77"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="70" t="s">
+      <c r="R2" s="120"/>
+      <c r="S2" s="120"/>
+      <c r="T2" s="121"/>
+    </row>
+    <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="129"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="136" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="71"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="64" t="s">
+      <c r="E3" s="137"/>
+      <c r="F3" s="138"/>
+      <c r="G3" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="99" t="s">
+      <c r="H3" s="131"/>
+      <c r="I3" s="131"/>
+      <c r="J3" s="131"/>
+      <c r="K3" s="132"/>
+      <c r="L3" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="100"/>
-      <c r="N3" s="100"/>
-      <c r="O3" s="100"/>
-      <c r="P3" s="101"/>
-      <c r="Q3" s="53" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="54"/>
-      <c r="S3" s="54"/>
-      <c r="T3" s="55"/>
-    </row>
-    <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="63"/>
-      <c r="B4" s="77"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="69"/>
-      <c r="L4" s="102"/>
-      <c r="M4" s="103"/>
-      <c r="N4" s="103"/>
-      <c r="O4" s="103"/>
-      <c r="P4" s="104"/>
-      <c r="Q4" s="56"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="58"/>
-    </row>
-    <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="63"/>
-      <c r="B5" s="77"/>
-      <c r="C5" s="79"/>
+      <c r="M3" s="114"/>
+      <c r="N3" s="114"/>
+      <c r="O3" s="114"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="122" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="123"/>
+      <c r="S3" s="123"/>
+      <c r="T3" s="124"/>
+    </row>
+    <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="129"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="139"/>
+      <c r="E4" s="140"/>
+      <c r="F4" s="141"/>
+      <c r="G4" s="133"/>
+      <c r="H4" s="134"/>
+      <c r="I4" s="134"/>
+      <c r="J4" s="134"/>
+      <c r="K4" s="135"/>
+      <c r="L4" s="116"/>
+      <c r="M4" s="117"/>
+      <c r="N4" s="117"/>
+      <c r="O4" s="117"/>
+      <c r="P4" s="118"/>
+      <c r="Q4" s="125"/>
+      <c r="R4" s="126"/>
+      <c r="S4" s="126"/>
+      <c r="T4" s="127"/>
+    </row>
+    <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="129"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="66"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -7276,7 +7280,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A6" s="10">
         <v>1</v>
       </c>
@@ -7318,7 +7322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A7" s="10">
         <v>2</v>
       </c>
@@ -7360,7 +7364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A8" s="10">
         <v>3</v>
       </c>
@@ -7402,7 +7406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A9" s="10">
         <v>4</v>
       </c>
@@ -7444,7 +7448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A10" s="10">
         <v>5</v>
       </c>
@@ -7486,7 +7490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A11" s="10">
         <v>6</v>
       </c>
@@ -7528,7 +7532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A12" s="10">
         <v>7</v>
       </c>
@@ -7570,7 +7574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A13" s="10">
         <v>8</v>
       </c>
@@ -7612,7 +7616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A14" s="10">
         <v>9</v>
       </c>
@@ -7654,7 +7658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A15" s="10">
         <v>10</v>
       </c>
@@ -7696,7 +7700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A16" s="10">
         <v>11</v>
       </c>
@@ -7738,7 +7742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A17" s="10">
         <v>12</v>
       </c>
@@ -7780,7 +7784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A18" s="10">
         <v>13</v>
       </c>
@@ -7822,7 +7826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A19" s="10">
         <v>14</v>
       </c>
@@ -7864,7 +7868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A20" s="10">
         <v>15</v>
       </c>
@@ -7906,7 +7910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A21" s="10">
         <v>16</v>
       </c>
@@ -7948,7 +7952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A22" s="10">
         <v>17</v>
       </c>
@@ -7990,7 +7994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A23" s="10">
         <v>18</v>
       </c>
@@ -8032,7 +8036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A24" s="10">
         <v>19</v>
       </c>
@@ -8074,7 +8078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A25" s="10">
         <v>20</v>
       </c>
@@ -8116,7 +8120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A26" s="10">
         <v>21</v>
       </c>
@@ -8158,7 +8162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A27" s="10">
         <v>22</v>
       </c>
@@ -8200,7 +8204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A28" s="10">
         <v>23</v>
       </c>
@@ -8242,7 +8246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A29" s="10">
         <v>24</v>
       </c>
@@ -8284,7 +8288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A30" s="10">
         <v>25</v>
       </c>
@@ -8326,7 +8330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A31" s="10">
         <v>26</v>
       </c>
@@ -8368,7 +8372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A32" s="10">
         <v>27</v>
       </c>
@@ -8410,7 +8414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A33" s="10">
         <v>28</v>
       </c>
@@ -8452,7 +8456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A34" s="10">
         <v>29</v>
       </c>
@@ -8494,7 +8498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A35" s="10">
         <v>30</v>
       </c>
@@ -8536,7 +8540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A36" s="10">
         <v>31</v>
       </c>
@@ -8578,7 +8582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A37" s="10">
         <v>32</v>
       </c>
@@ -8620,7 +8624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A38" s="10">
         <v>33</v>
       </c>
@@ -8662,7 +8666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A39" s="10">
         <v>34</v>
       </c>
@@ -8704,7 +8708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A40" s="10">
         <v>35</v>
       </c>
@@ -8746,7 +8750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A41" s="10">
         <v>36</v>
       </c>
@@ -8788,7 +8792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A42" s="10">
         <v>37</v>
       </c>
@@ -8830,7 +8834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A43" s="10">
         <v>38</v>
       </c>
@@ -8872,7 +8876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A44" s="10">
         <v>39</v>
       </c>
@@ -8914,7 +8918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A45" s="10">
         <v>40</v>
       </c>
@@ -8956,7 +8960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A46" s="10">
         <v>41</v>
       </c>
@@ -8998,7 +9002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A47" s="10">
         <v>42</v>
       </c>
@@ -9040,7 +9044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A48" s="10">
         <v>43</v>
       </c>
@@ -9082,7 +9086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A49" s="10">
         <v>44</v>
       </c>
@@ -9124,7 +9128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A50" s="10">
         <v>45</v>
       </c>
@@ -9166,7 +9170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A51" s="10">
         <v>46</v>
       </c>
@@ -9208,7 +9212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A52" s="10">
         <v>47</v>
       </c>
@@ -9250,7 +9254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A53" s="10">
         <v>48</v>
       </c>
@@ -9292,7 +9296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A54" s="10">
         <v>49</v>
       </c>
@@ -9334,7 +9338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A55" s="10">
         <v>50</v>
       </c>
@@ -9376,7 +9380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A56" s="10">
         <v>51</v>
       </c>
@@ -9418,7 +9422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A57" s="10">
         <v>52</v>
       </c>
@@ -9460,7 +9464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A58" s="10">
         <v>53</v>
       </c>
@@ -9502,7 +9506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A59" s="10">
         <v>54</v>
       </c>
@@ -9544,7 +9548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A60" s="10">
         <v>55</v>
       </c>
@@ -9586,7 +9590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A61" s="10">
         <v>56</v>
       </c>
@@ -9628,7 +9632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A62" s="10">
         <v>57</v>
       </c>
@@ -9670,7 +9674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:20" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A63" s="10">
         <v>58</v>
       </c>
@@ -9712,7 +9716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="20.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="10">
         <v>59</v>
       </c>
@@ -9754,184 +9758,193 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D65" s="84" t="s">
+    <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D65" s="95" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="87" t="s">
+      <c r="E65" s="98" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="81" t="s">
+      <c r="G65" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="93" t="s">
+      <c r="H65" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="93" t="s">
+      <c r="I65" s="107" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="81" t="s">
+      <c r="J65" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="59" t="s">
+      <c r="L65" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="90" t="s">
+      <c r="M65" s="104" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="90" t="s">
+      <c r="N65" s="104" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="59" t="s">
+      <c r="O65" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="96" t="s">
+      <c r="Q65" s="110" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="96" t="s">
+      <c r="R65" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="96" t="s">
+      <c r="S65" s="110" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D66" s="85"/>
-      <c r="E66" s="88"/>
-      <c r="G66" s="82"/>
-      <c r="H66" s="94"/>
-      <c r="I66" s="94"/>
-      <c r="J66" s="82"/>
-      <c r="L66" s="60"/>
-      <c r="M66" s="91"/>
-      <c r="N66" s="91"/>
-      <c r="O66" s="60"/>
-      <c r="Q66" s="97"/>
-      <c r="R66" s="97"/>
-      <c r="S66" s="97"/>
-    </row>
-    <row r="67" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D67" s="85"/>
-      <c r="E67" s="88"/>
-      <c r="G67" s="82"/>
-      <c r="H67" s="94"/>
-      <c r="I67" s="94"/>
-      <c r="J67" s="82"/>
-      <c r="L67" s="60"/>
-      <c r="M67" s="91"/>
-      <c r="N67" s="91"/>
-      <c r="O67" s="60"/>
-      <c r="Q67" s="97"/>
-      <c r="R67" s="97"/>
-      <c r="S67" s="97"/>
-    </row>
-    <row r="68" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D68" s="85"/>
-      <c r="E68" s="88"/>
-      <c r="G68" s="82"/>
-      <c r="H68" s="94"/>
-      <c r="I68" s="94"/>
-      <c r="J68" s="82"/>
-      <c r="L68" s="60"/>
-      <c r="M68" s="91"/>
-      <c r="N68" s="91"/>
-      <c r="O68" s="60"/>
-      <c r="Q68" s="97"/>
-      <c r="R68" s="97"/>
-      <c r="S68" s="97"/>
-    </row>
-    <row r="69" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D69" s="85"/>
-      <c r="E69" s="88"/>
-      <c r="G69" s="82"/>
-      <c r="H69" s="94"/>
-      <c r="I69" s="94"/>
-      <c r="J69" s="82"/>
-      <c r="L69" s="60"/>
-      <c r="M69" s="91"/>
-      <c r="N69" s="91"/>
-      <c r="O69" s="60"/>
-      <c r="Q69" s="97"/>
-      <c r="R69" s="97"/>
-      <c r="S69" s="97"/>
-    </row>
-    <row r="70" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D70" s="85"/>
-      <c r="E70" s="88"/>
-      <c r="G70" s="82"/>
-      <c r="H70" s="94"/>
-      <c r="I70" s="94"/>
-      <c r="J70" s="82"/>
-      <c r="L70" s="60"/>
-      <c r="M70" s="91"/>
-      <c r="N70" s="91"/>
-      <c r="O70" s="60"/>
-      <c r="Q70" s="97"/>
-      <c r="R70" s="97"/>
-      <c r="S70" s="97"/>
-    </row>
-    <row r="71" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D71" s="85"/>
-      <c r="E71" s="88"/>
-      <c r="G71" s="82"/>
-      <c r="H71" s="94"/>
-      <c r="I71" s="94"/>
-      <c r="J71" s="82"/>
-      <c r="L71" s="60"/>
-      <c r="M71" s="91"/>
-      <c r="N71" s="91"/>
-      <c r="O71" s="60"/>
-      <c r="Q71" s="97"/>
-      <c r="R71" s="97"/>
-      <c r="S71" s="97"/>
-    </row>
-    <row r="72" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D72" s="85"/>
-      <c r="E72" s="88"/>
-      <c r="G72" s="82"/>
-      <c r="H72" s="94"/>
-      <c r="I72" s="94"/>
-      <c r="J72" s="82"/>
-      <c r="L72" s="60"/>
-      <c r="M72" s="91"/>
-      <c r="N72" s="91"/>
-      <c r="O72" s="60"/>
-      <c r="Q72" s="97"/>
-      <c r="R72" s="97"/>
-      <c r="S72" s="97"/>
-    </row>
-    <row r="73" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D73" s="85"/>
-      <c r="E73" s="88"/>
-      <c r="G73" s="82"/>
-      <c r="H73" s="94"/>
-      <c r="I73" s="94"/>
-      <c r="J73" s="82"/>
-      <c r="L73" s="60"/>
-      <c r="M73" s="91"/>
-      <c r="N73" s="91"/>
-      <c r="O73" s="60"/>
-      <c r="Q73" s="97"/>
-      <c r="R73" s="97"/>
-      <c r="S73" s="97"/>
-    </row>
-    <row r="74" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D74" s="86"/>
-      <c r="E74" s="89"/>
-      <c r="G74" s="83"/>
-      <c r="H74" s="95"/>
-      <c r="I74" s="95"/>
-      <c r="J74" s="83"/>
-      <c r="L74" s="61"/>
-      <c r="M74" s="92"/>
-      <c r="N74" s="92"/>
-      <c r="O74" s="61"/>
-      <c r="Q74" s="98"/>
-      <c r="R74" s="98"/>
-      <c r="S74" s="98"/>
+    <row r="66" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D66" s="96"/>
+      <c r="E66" s="99"/>
+      <c r="G66" s="93"/>
+      <c r="H66" s="108"/>
+      <c r="I66" s="108"/>
+      <c r="J66" s="93"/>
+      <c r="L66" s="102"/>
+      <c r="M66" s="105"/>
+      <c r="N66" s="105"/>
+      <c r="O66" s="102"/>
+      <c r="Q66" s="111"/>
+      <c r="R66" s="111"/>
+      <c r="S66" s="111"/>
+    </row>
+    <row r="67" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D67" s="96"/>
+      <c r="E67" s="99"/>
+      <c r="G67" s="93"/>
+      <c r="H67" s="108"/>
+      <c r="I67" s="108"/>
+      <c r="J67" s="93"/>
+      <c r="L67" s="102"/>
+      <c r="M67" s="105"/>
+      <c r="N67" s="105"/>
+      <c r="O67" s="102"/>
+      <c r="Q67" s="111"/>
+      <c r="R67" s="111"/>
+      <c r="S67" s="111"/>
+    </row>
+    <row r="68" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D68" s="96"/>
+      <c r="E68" s="99"/>
+      <c r="G68" s="93"/>
+      <c r="H68" s="108"/>
+      <c r="I68" s="108"/>
+      <c r="J68" s="93"/>
+      <c r="L68" s="102"/>
+      <c r="M68" s="105"/>
+      <c r="N68" s="105"/>
+      <c r="O68" s="102"/>
+      <c r="Q68" s="111"/>
+      <c r="R68" s="111"/>
+      <c r="S68" s="111"/>
+    </row>
+    <row r="69" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D69" s="96"/>
+      <c r="E69" s="99"/>
+      <c r="G69" s="93"/>
+      <c r="H69" s="108"/>
+      <c r="I69" s="108"/>
+      <c r="J69" s="93"/>
+      <c r="L69" s="102"/>
+      <c r="M69" s="105"/>
+      <c r="N69" s="105"/>
+      <c r="O69" s="102"/>
+      <c r="Q69" s="111"/>
+      <c r="R69" s="111"/>
+      <c r="S69" s="111"/>
+    </row>
+    <row r="70" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D70" s="96"/>
+      <c r="E70" s="99"/>
+      <c r="G70" s="93"/>
+      <c r="H70" s="108"/>
+      <c r="I70" s="108"/>
+      <c r="J70" s="93"/>
+      <c r="L70" s="102"/>
+      <c r="M70" s="105"/>
+      <c r="N70" s="105"/>
+      <c r="O70" s="102"/>
+      <c r="Q70" s="111"/>
+      <c r="R70" s="111"/>
+      <c r="S70" s="111"/>
+    </row>
+    <row r="71" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D71" s="96"/>
+      <c r="E71" s="99"/>
+      <c r="G71" s="93"/>
+      <c r="H71" s="108"/>
+      <c r="I71" s="108"/>
+      <c r="J71" s="93"/>
+      <c r="L71" s="102"/>
+      <c r="M71" s="105"/>
+      <c r="N71" s="105"/>
+      <c r="O71" s="102"/>
+      <c r="Q71" s="111"/>
+      <c r="R71" s="111"/>
+      <c r="S71" s="111"/>
+    </row>
+    <row r="72" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D72" s="96"/>
+      <c r="E72" s="99"/>
+      <c r="G72" s="93"/>
+      <c r="H72" s="108"/>
+      <c r="I72" s="108"/>
+      <c r="J72" s="93"/>
+      <c r="L72" s="102"/>
+      <c r="M72" s="105"/>
+      <c r="N72" s="105"/>
+      <c r="O72" s="102"/>
+      <c r="Q72" s="111"/>
+      <c r="R72" s="111"/>
+      <c r="S72" s="111"/>
+    </row>
+    <row r="73" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D73" s="96"/>
+      <c r="E73" s="99"/>
+      <c r="G73" s="93"/>
+      <c r="H73" s="108"/>
+      <c r="I73" s="108"/>
+      <c r="J73" s="93"/>
+      <c r="L73" s="102"/>
+      <c r="M73" s="105"/>
+      <c r="N73" s="105"/>
+      <c r="O73" s="102"/>
+      <c r="Q73" s="111"/>
+      <c r="R73" s="111"/>
+      <c r="S73" s="111"/>
+    </row>
+    <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D74" s="97"/>
+      <c r="E74" s="100"/>
+      <c r="G74" s="94"/>
+      <c r="H74" s="109"/>
+      <c r="I74" s="109"/>
+      <c r="J74" s="94"/>
+      <c r="L74" s="103"/>
+      <c r="M74" s="106"/>
+      <c r="N74" s="106"/>
+      <c r="O74" s="103"/>
+      <c r="Q74" s="112"/>
+      <c r="R74" s="112"/>
+      <c r="S74" s="112"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9948,15 +9961,6 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
pregunta 7 mejor resuelta y representada
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F5D2C8-6DF9-4556-A98E-E83C72C23806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{151A41F0-26B8-4648-9255-776CEB5B86C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1271,7 +1271,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1425,6 +1425,9 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1539,6 +1542,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1569,15 +1650,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1623,79 +1695,8 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -2202,28 +2203,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="57"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -2413,11 +2414,11 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="142">
+      <c r="A10" s="53">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B10" s="143" t="s">
+      <c r="B10" s="144" t="s">
         <v>64</v>
       </c>
       <c r="C10" s="50" t="s">
@@ -2444,7 +2445,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B11" s="143" t="s">
+      <c r="B11" s="144" t="s">
         <v>158</v>
       </c>
       <c r="C11" s="50" t="s">
@@ -2471,7 +2472,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B12" s="143" t="s">
+      <c r="B12" s="144" t="s">
         <v>236</v>
       </c>
       <c r="C12" s="50" t="s">
@@ -2498,7 +2499,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B13" s="143" t="s">
+      <c r="B13" s="144" t="s">
         <v>186</v>
       </c>
       <c r="C13" s="50" t="s">
@@ -2525,7 +2526,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B14" s="143" t="s">
+      <c r="B14" s="144" t="s">
         <v>138</v>
       </c>
       <c r="C14" s="50" t="s">
@@ -2552,7 +2553,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B15" s="143" t="s">
+      <c r="B15" s="144" t="s">
         <v>100</v>
       </c>
       <c r="C15" s="50" t="s">
@@ -2579,7 +2580,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B16" s="50" t="s">
+      <c r="B16" s="143" t="s">
         <v>86</v>
       </c>
       <c r="C16" s="50" t="s">
@@ -2606,7 +2607,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="143" t="s">
         <v>219</v>
       </c>
       <c r="C17" s="50" t="s">
@@ -2633,7 +2634,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B18" s="50" t="s">
+      <c r="B18" s="143" t="s">
         <v>251</v>
       </c>
       <c r="C18" s="50" t="s">
@@ -2660,7 +2661,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B19" s="50" t="s">
+      <c r="B19" s="143" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="50" t="s">
@@ -2687,7 +2688,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B20" s="50" t="s">
+      <c r="B20" s="143" t="s">
         <v>55</v>
       </c>
       <c r="C20" s="50" t="s">
@@ -2714,7 +2715,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B21" s="50" t="s">
+      <c r="B21" s="143" t="s">
         <v>114</v>
       </c>
       <c r="C21" s="50" t="s">
@@ -3732,172 +3733,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="64"/>
-      <c r="S1" s="64"/>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="64"/>
-      <c r="W1" s="64"/>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="64"/>
-      <c r="AC1" s="64"/>
-      <c r="AD1" s="64"/>
-      <c r="AE1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="65"/>
+      <c r="V1" s="65"/>
+      <c r="W1" s="65"/>
+      <c r="X1" s="65"/>
+      <c r="Y1" s="65"/>
+      <c r="Z1" s="65"/>
+      <c r="AA1" s="65"/>
+      <c r="AB1" s="65"/>
+      <c r="AC1" s="65"/>
+      <c r="AD1" s="65"/>
+      <c r="AE1" s="65"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="82" t="s">
+      <c r="D2" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="67" t="s">
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="76" t="s">
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="77"/>
-      <c r="T2" s="77"/>
-      <c r="U2" s="77"/>
-      <c r="V2" s="77"/>
-      <c r="W2" s="77"/>
-      <c r="X2" s="77"/>
-      <c r="Y2" s="77"/>
-      <c r="Z2" s="78"/>
-      <c r="AA2" s="57" t="s">
+      <c r="S2" s="78"/>
+      <c r="T2" s="78"/>
+      <c r="U2" s="78"/>
+      <c r="V2" s="78"/>
+      <c r="W2" s="78"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="78"/>
+      <c r="Z2" s="79"/>
+      <c r="AA2" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="58"/>
-      <c r="AC2" s="58"/>
-      <c r="AD2" s="58"/>
-      <c r="AE2" s="59"/>
+      <c r="AB2" s="59"/>
+      <c r="AC2" s="59"/>
+      <c r="AD2" s="59"/>
+      <c r="AE2" s="60"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="66"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="85" t="s">
+      <c r="A3" s="67"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="70" t="s">
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="71"/>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="79" t="s">
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
+      <c r="L3" s="72"/>
+      <c r="M3" s="72"/>
+      <c r="N3" s="72"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="72"/>
+      <c r="Q3" s="73"/>
+      <c r="R3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="80"/>
-      <c r="T3" s="80"/>
-      <c r="U3" s="80"/>
-      <c r="V3" s="80"/>
-      <c r="W3" s="80"/>
-      <c r="X3" s="80"/>
-      <c r="Y3" s="80"/>
-      <c r="Z3" s="81"/>
-      <c r="AA3" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="61"/>
-      <c r="AC3" s="61"/>
-      <c r="AD3" s="61"/>
-      <c r="AE3" s="62"/>
+      <c r="S3" s="81"/>
+      <c r="T3" s="81"/>
+      <c r="U3" s="81"/>
+      <c r="V3" s="81"/>
+      <c r="W3" s="81"/>
+      <c r="X3" s="81"/>
+      <c r="Y3" s="81"/>
+      <c r="Z3" s="82"/>
+      <c r="AA3" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="62"/>
+      <c r="AC3" s="62"/>
+      <c r="AD3" s="62"/>
+      <c r="AE3" s="63"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="88" t="s">
+      <c r="A4" s="67"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="89" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="75"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="76"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="73" t="s">
+      <c r="I4" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
-      <c r="M4" s="74"/>
-      <c r="N4" s="74"/>
-      <c r="O4" s="74"/>
-      <c r="P4" s="75"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="75"/>
+      <c r="N4" s="75"/>
+      <c r="O4" s="75"/>
+      <c r="P4" s="76"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="73" t="s">
+      <c r="R4" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="74"/>
-      <c r="T4" s="74"/>
-      <c r="U4" s="74"/>
-      <c r="V4" s="74"/>
-      <c r="W4" s="74"/>
-      <c r="X4" s="74"/>
-      <c r="Y4" s="75"/>
+      <c r="S4" s="75"/>
+      <c r="T4" s="75"/>
+      <c r="U4" s="75"/>
+      <c r="V4" s="75"/>
+      <c r="W4" s="75"/>
+      <c r="X4" s="75"/>
+      <c r="Y4" s="76"/>
       <c r="Z4" s="13"/>
-      <c r="AA4" s="63" t="s">
+      <c r="AA4" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="AB4" s="63"/>
-      <c r="AC4" s="63"/>
-      <c r="AD4" s="63"/>
+      <c r="AB4" s="64"/>
+      <c r="AC4" s="64"/>
+      <c r="AD4" s="64"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="66"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="66"/>
+      <c r="A5" s="67"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="34"/>
       <c r="E5" s="34"/>
       <c r="F5" s="34"/>
@@ -7111,123 +7112,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="91" t="s">
+      <c r="B1" s="118" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="91"/>
-      <c r="L1" s="91"/>
-      <c r="M1" s="91"/>
-      <c r="N1" s="91"/>
-      <c r="O1" s="91"/>
-      <c r="P1" s="91"/>
-      <c r="Q1" s="91"/>
-      <c r="R1" s="91"/>
-      <c r="S1" s="91"/>
-      <c r="T1" s="91"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="118"/>
+      <c r="J1" s="118"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
+      <c r="P1" s="118"/>
+      <c r="Q1" s="118"/>
+      <c r="R1" s="118"/>
+      <c r="S1" s="118"/>
+      <c r="T1" s="118"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="119" t="str">
+      <c r="D2" s="92" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="120"/>
-      <c r="F2" s="121"/>
-      <c r="G2" s="119" t="str">
+      <c r="E2" s="93"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="92" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="121"/>
-      <c r="L2" s="119" t="s">
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="120"/>
-      <c r="N2" s="120"/>
-      <c r="O2" s="120"/>
-      <c r="P2" s="121"/>
-      <c r="Q2" s="119" t="str">
+      <c r="M2" s="93"/>
+      <c r="N2" s="93"/>
+      <c r="O2" s="93"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="92" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="120"/>
-      <c r="S2" s="120"/>
-      <c r="T2" s="121"/>
+      <c r="R2" s="93"/>
+      <c r="S2" s="93"/>
+      <c r="T2" s="94"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="129"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="136" t="s">
+      <c r="A3" s="105"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="112" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="137"/>
-      <c r="F3" s="138"/>
-      <c r="G3" s="130" t="s">
+      <c r="E3" s="113"/>
+      <c r="F3" s="114"/>
+      <c r="G3" s="106" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="131"/>
-      <c r="I3" s="131"/>
-      <c r="J3" s="131"/>
-      <c r="K3" s="132"/>
-      <c r="L3" s="113" t="s">
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="108"/>
+      <c r="L3" s="137" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="114"/>
-      <c r="N3" s="114"/>
-      <c r="O3" s="114"/>
-      <c r="P3" s="115"/>
-      <c r="Q3" s="122" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="123"/>
-      <c r="S3" s="123"/>
-      <c r="T3" s="124"/>
+      <c r="M3" s="138"/>
+      <c r="N3" s="138"/>
+      <c r="O3" s="138"/>
+      <c r="P3" s="139"/>
+      <c r="Q3" s="95" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="96"/>
+      <c r="S3" s="96"/>
+      <c r="T3" s="97"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="129"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="139"/>
-      <c r="E4" s="140"/>
-      <c r="F4" s="141"/>
-      <c r="G4" s="133"/>
-      <c r="H4" s="134"/>
-      <c r="I4" s="134"/>
-      <c r="J4" s="134"/>
-      <c r="K4" s="135"/>
-      <c r="L4" s="116"/>
-      <c r="M4" s="117"/>
-      <c r="N4" s="117"/>
-      <c r="O4" s="117"/>
-      <c r="P4" s="118"/>
-      <c r="Q4" s="125"/>
-      <c r="R4" s="126"/>
-      <c r="S4" s="126"/>
-      <c r="T4" s="127"/>
+      <c r="A4" s="105"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="115"/>
+      <c r="E4" s="116"/>
+      <c r="F4" s="117"/>
+      <c r="G4" s="109"/>
+      <c r="H4" s="110"/>
+      <c r="I4" s="110"/>
+      <c r="J4" s="110"/>
+      <c r="K4" s="111"/>
+      <c r="L4" s="140"/>
+      <c r="M4" s="141"/>
+      <c r="N4" s="141"/>
+      <c r="O4" s="141"/>
+      <c r="P4" s="142"/>
+      <c r="Q4" s="98"/>
+      <c r="R4" s="99"/>
+      <c r="S4" s="99"/>
+      <c r="T4" s="100"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="129"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="66"/>
+      <c r="A5" s="105"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9759,192 +9760,183 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="95" t="s">
+      <c r="D65" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="98" t="s">
+      <c r="E65" s="125" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="92" t="s">
+      <c r="G65" s="119" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="107" t="s">
+      <c r="H65" s="131" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="107" t="s">
+      <c r="I65" s="131" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="92" t="s">
+      <c r="J65" s="119" t="s">
         <v>11</v>
       </c>
       <c r="L65" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="104" t="s">
+      <c r="M65" s="128" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="104" t="s">
+      <c r="N65" s="128" t="s">
         <v>10</v>
       </c>
       <c r="O65" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="110" t="s">
+      <c r="Q65" s="134" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="110" t="s">
+      <c r="R65" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="110" t="s">
+      <c r="S65" s="134" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="96"/>
-      <c r="E66" s="99"/>
-      <c r="G66" s="93"/>
-      <c r="H66" s="108"/>
-      <c r="I66" s="108"/>
-      <c r="J66" s="93"/>
+      <c r="D66" s="123"/>
+      <c r="E66" s="126"/>
+      <c r="G66" s="120"/>
+      <c r="H66" s="132"/>
+      <c r="I66" s="132"/>
+      <c r="J66" s="120"/>
       <c r="L66" s="102"/>
-      <c r="M66" s="105"/>
-      <c r="N66" s="105"/>
+      <c r="M66" s="129"/>
+      <c r="N66" s="129"/>
       <c r="O66" s="102"/>
-      <c r="Q66" s="111"/>
-      <c r="R66" s="111"/>
-      <c r="S66" s="111"/>
+      <c r="Q66" s="135"/>
+      <c r="R66" s="135"/>
+      <c r="S66" s="135"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="96"/>
-      <c r="E67" s="99"/>
-      <c r="G67" s="93"/>
-      <c r="H67" s="108"/>
-      <c r="I67" s="108"/>
-      <c r="J67" s="93"/>
+      <c r="D67" s="123"/>
+      <c r="E67" s="126"/>
+      <c r="G67" s="120"/>
+      <c r="H67" s="132"/>
+      <c r="I67" s="132"/>
+      <c r="J67" s="120"/>
       <c r="L67" s="102"/>
-      <c r="M67" s="105"/>
-      <c r="N67" s="105"/>
+      <c r="M67" s="129"/>
+      <c r="N67" s="129"/>
       <c r="O67" s="102"/>
-      <c r="Q67" s="111"/>
-      <c r="R67" s="111"/>
-      <c r="S67" s="111"/>
+      <c r="Q67" s="135"/>
+      <c r="R67" s="135"/>
+      <c r="S67" s="135"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="96"/>
-      <c r="E68" s="99"/>
-      <c r="G68" s="93"/>
-      <c r="H68" s="108"/>
-      <c r="I68" s="108"/>
-      <c r="J68" s="93"/>
+      <c r="D68" s="123"/>
+      <c r="E68" s="126"/>
+      <c r="G68" s="120"/>
+      <c r="H68" s="132"/>
+      <c r="I68" s="132"/>
+      <c r="J68" s="120"/>
       <c r="L68" s="102"/>
-      <c r="M68" s="105"/>
-      <c r="N68" s="105"/>
+      <c r="M68" s="129"/>
+      <c r="N68" s="129"/>
       <c r="O68" s="102"/>
-      <c r="Q68" s="111"/>
-      <c r="R68" s="111"/>
-      <c r="S68" s="111"/>
+      <c r="Q68" s="135"/>
+      <c r="R68" s="135"/>
+      <c r="S68" s="135"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="96"/>
-      <c r="E69" s="99"/>
-      <c r="G69" s="93"/>
-      <c r="H69" s="108"/>
-      <c r="I69" s="108"/>
-      <c r="J69" s="93"/>
+      <c r="D69" s="123"/>
+      <c r="E69" s="126"/>
+      <c r="G69" s="120"/>
+      <c r="H69" s="132"/>
+      <c r="I69" s="132"/>
+      <c r="J69" s="120"/>
       <c r="L69" s="102"/>
-      <c r="M69" s="105"/>
-      <c r="N69" s="105"/>
+      <c r="M69" s="129"/>
+      <c r="N69" s="129"/>
       <c r="O69" s="102"/>
-      <c r="Q69" s="111"/>
-      <c r="R69" s="111"/>
-      <c r="S69" s="111"/>
+      <c r="Q69" s="135"/>
+      <c r="R69" s="135"/>
+      <c r="S69" s="135"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="96"/>
-      <c r="E70" s="99"/>
-      <c r="G70" s="93"/>
-      <c r="H70" s="108"/>
-      <c r="I70" s="108"/>
-      <c r="J70" s="93"/>
+      <c r="D70" s="123"/>
+      <c r="E70" s="126"/>
+      <c r="G70" s="120"/>
+      <c r="H70" s="132"/>
+      <c r="I70" s="132"/>
+      <c r="J70" s="120"/>
       <c r="L70" s="102"/>
-      <c r="M70" s="105"/>
-      <c r="N70" s="105"/>
+      <c r="M70" s="129"/>
+      <c r="N70" s="129"/>
       <c r="O70" s="102"/>
-      <c r="Q70" s="111"/>
-      <c r="R70" s="111"/>
-      <c r="S70" s="111"/>
+      <c r="Q70" s="135"/>
+      <c r="R70" s="135"/>
+      <c r="S70" s="135"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="96"/>
-      <c r="E71" s="99"/>
-      <c r="G71" s="93"/>
-      <c r="H71" s="108"/>
-      <c r="I71" s="108"/>
-      <c r="J71" s="93"/>
+      <c r="D71" s="123"/>
+      <c r="E71" s="126"/>
+      <c r="G71" s="120"/>
+      <c r="H71" s="132"/>
+      <c r="I71" s="132"/>
+      <c r="J71" s="120"/>
       <c r="L71" s="102"/>
-      <c r="M71" s="105"/>
-      <c r="N71" s="105"/>
+      <c r="M71" s="129"/>
+      <c r="N71" s="129"/>
       <c r="O71" s="102"/>
-      <c r="Q71" s="111"/>
-      <c r="R71" s="111"/>
-      <c r="S71" s="111"/>
+      <c r="Q71" s="135"/>
+      <c r="R71" s="135"/>
+      <c r="S71" s="135"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="96"/>
-      <c r="E72" s="99"/>
-      <c r="G72" s="93"/>
-      <c r="H72" s="108"/>
-      <c r="I72" s="108"/>
-      <c r="J72" s="93"/>
+      <c r="D72" s="123"/>
+      <c r="E72" s="126"/>
+      <c r="G72" s="120"/>
+      <c r="H72" s="132"/>
+      <c r="I72" s="132"/>
+      <c r="J72" s="120"/>
       <c r="L72" s="102"/>
-      <c r="M72" s="105"/>
-      <c r="N72" s="105"/>
+      <c r="M72" s="129"/>
+      <c r="N72" s="129"/>
       <c r="O72" s="102"/>
-      <c r="Q72" s="111"/>
-      <c r="R72" s="111"/>
-      <c r="S72" s="111"/>
+      <c r="Q72" s="135"/>
+      <c r="R72" s="135"/>
+      <c r="S72" s="135"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="96"/>
-      <c r="E73" s="99"/>
-      <c r="G73" s="93"/>
-      <c r="H73" s="108"/>
-      <c r="I73" s="108"/>
-      <c r="J73" s="93"/>
+      <c r="D73" s="123"/>
+      <c r="E73" s="126"/>
+      <c r="G73" s="120"/>
+      <c r="H73" s="132"/>
+      <c r="I73" s="132"/>
+      <c r="J73" s="120"/>
       <c r="L73" s="102"/>
-      <c r="M73" s="105"/>
-      <c r="N73" s="105"/>
+      <c r="M73" s="129"/>
+      <c r="N73" s="129"/>
       <c r="O73" s="102"/>
-      <c r="Q73" s="111"/>
-      <c r="R73" s="111"/>
-      <c r="S73" s="111"/>
+      <c r="Q73" s="135"/>
+      <c r="R73" s="135"/>
+      <c r="S73" s="135"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="97"/>
-      <c r="E74" s="100"/>
-      <c r="G74" s="94"/>
-      <c r="H74" s="109"/>
-      <c r="I74" s="109"/>
-      <c r="J74" s="94"/>
+      <c r="D74" s="124"/>
+      <c r="E74" s="127"/>
+      <c r="G74" s="121"/>
+      <c r="H74" s="133"/>
+      <c r="I74" s="133"/>
+      <c r="J74" s="121"/>
       <c r="L74" s="103"/>
-      <c r="M74" s="106"/>
-      <c r="N74" s="106"/>
+      <c r="M74" s="130"/>
+      <c r="N74" s="130"/>
       <c r="O74" s="103"/>
-      <c r="Q74" s="112"/>
-      <c r="R74" s="112"/>
-      <c r="S74" s="112"/>
+      <c r="Q74" s="136"/>
+      <c r="R74" s="136"/>
+      <c r="S74" s="136"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9961,6 +9953,15 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
debemos generar y promocionar los recursos.
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25769CC-EF86-4DFF-AA77-49870A16F637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5459A84D-E359-408E-A240-65C83EEF8EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -983,7 +983,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1053,6 +1053,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1271,7 +1277,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1540,6 +1546,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1570,15 +1654,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1624,80 +1699,8 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -2415,7 +2418,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="145">
+      <c r="A10" s="44">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -2581,7 +2584,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B16" s="144" t="s">
+      <c r="B16" s="53" t="s">
         <v>86</v>
       </c>
       <c r="C16" s="50" t="s">
@@ -2608,7 +2611,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B17" s="144" t="s">
+      <c r="B17" s="53" t="s">
         <v>219</v>
       </c>
       <c r="C17" s="50" t="s">
@@ -2635,7 +2638,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B18" s="144" t="s">
+      <c r="B18" s="53" t="s">
         <v>251</v>
       </c>
       <c r="C18" s="50" t="s">
@@ -2662,7 +2665,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B19" s="144" t="s">
+      <c r="B19" s="53" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="50" t="s">
@@ -2689,7 +2692,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B20" s="144" t="s">
+      <c r="B20" s="53" t="s">
         <v>55</v>
       </c>
       <c r="C20" s="50" t="s">
@@ -2716,7 +2719,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B21" s="144" t="s">
+      <c r="B21" s="53" t="s">
         <v>114</v>
       </c>
       <c r="C21" s="50" t="s">
@@ -2743,7 +2746,7 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B22" s="144" t="s">
+      <c r="B22" s="53" t="s">
         <v>124</v>
       </c>
       <c r="C22" s="50" t="s">
@@ -2770,7 +2773,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B23" s="143" t="s">
+      <c r="B23" s="144" t="s">
         <v>167</v>
       </c>
       <c r="C23" s="50" t="s">
@@ -2797,7 +2800,7 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B24" s="143" t="s">
+      <c r="B24" s="144" t="s">
         <v>199</v>
       </c>
       <c r="C24" s="50" t="s">
@@ -2824,7 +2827,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B25" s="143" t="s">
+      <c r="B25" s="144" t="s">
         <v>69</v>
       </c>
       <c r="C25" s="50" t="s">
@@ -2851,7 +2854,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="B26" s="143" t="s">
+      <c r="B26" s="144" t="s">
         <v>241</v>
       </c>
       <c r="C26" s="50" t="s">
@@ -2878,7 +2881,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="B27" s="143" t="s">
+      <c r="B27" s="144" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="50" t="s">
@@ -2905,7 +2908,7 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="B28" s="143" t="s">
+      <c r="B28" s="144" t="s">
         <v>77</v>
       </c>
       <c r="C28" s="50" t="s">
@@ -2932,7 +2935,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B29" s="143" t="s">
+      <c r="B29" s="144" t="s">
         <v>246</v>
       </c>
       <c r="C29" s="50" t="s">
@@ -2959,7 +2962,7 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="B30" s="50" t="s">
+      <c r="B30" s="143" t="s">
         <v>223</v>
       </c>
       <c r="C30" s="50" t="s">
@@ -2986,7 +2989,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B31" s="50" t="s">
+      <c r="B31" s="143" t="s">
         <v>207</v>
       </c>
       <c r="C31" s="50" t="s">
@@ -3013,7 +3016,7 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="B32" s="50" t="s">
+      <c r="B32" s="143" t="s">
         <v>211</v>
       </c>
       <c r="C32" s="50" t="s">
@@ -3040,7 +3043,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B33" s="50" t="s">
+      <c r="B33" s="143" t="s">
         <v>215</v>
       </c>
       <c r="C33" s="50" t="s">
@@ -3067,7 +3070,7 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="B34" s="50" t="s">
+      <c r="B34" s="143" t="s">
         <v>227</v>
       </c>
       <c r="C34" s="50" t="s">
@@ -3094,7 +3097,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B35" s="50" t="s">
+      <c r="B35" s="143" t="s">
         <v>73</v>
       </c>
       <c r="C35" s="50" t="s">
@@ -7113,30 +7116,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="118" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="92"/>
-      <c r="T1" s="92"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="118"/>
+      <c r="J1" s="118"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
+      <c r="P1" s="118"/>
+      <c r="Q1" s="118"/>
+      <c r="R1" s="118"/>
+      <c r="S1" s="118"/>
+      <c r="T1" s="118"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="104" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="90" t="s">
@@ -7145,89 +7148,89 @@
       <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="120" t="str">
+      <c r="D2" s="92" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="121"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="120" t="str">
+      <c r="E2" s="93"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="92" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="121"/>
-      <c r="I2" s="121"/>
-      <c r="J2" s="121"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="120" t="s">
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="121"/>
-      <c r="N2" s="121"/>
-      <c r="O2" s="121"/>
-      <c r="P2" s="122"/>
-      <c r="Q2" s="120" t="str">
+      <c r="M2" s="93"/>
+      <c r="N2" s="93"/>
+      <c r="O2" s="93"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="92" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="121"/>
-      <c r="S2" s="121"/>
-      <c r="T2" s="122"/>
+      <c r="R2" s="93"/>
+      <c r="S2" s="93"/>
+      <c r="T2" s="94"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="130"/>
+      <c r="A3" s="105"/>
       <c r="B3" s="91"/>
       <c r="C3" s="67"/>
-      <c r="D3" s="137" t="s">
+      <c r="D3" s="112" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="138"/>
-      <c r="F3" s="139"/>
-      <c r="G3" s="131" t="s">
+      <c r="E3" s="113"/>
+      <c r="F3" s="114"/>
+      <c r="G3" s="106" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="132"/>
-      <c r="I3" s="132"/>
-      <c r="J3" s="132"/>
-      <c r="K3" s="133"/>
-      <c r="L3" s="114" t="s">
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="108"/>
+      <c r="L3" s="137" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="115"/>
-      <c r="N3" s="115"/>
-      <c r="O3" s="115"/>
-      <c r="P3" s="116"/>
-      <c r="Q3" s="123" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="124"/>
-      <c r="S3" s="124"/>
-      <c r="T3" s="125"/>
+      <c r="M3" s="138"/>
+      <c r="N3" s="138"/>
+      <c r="O3" s="138"/>
+      <c r="P3" s="139"/>
+      <c r="Q3" s="95" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="96"/>
+      <c r="S3" s="96"/>
+      <c r="T3" s="97"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="130"/>
+      <c r="A4" s="105"/>
       <c r="B4" s="91"/>
       <c r="C4" s="67"/>
-      <c r="D4" s="140"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="142"/>
-      <c r="G4" s="134"/>
-      <c r="H4" s="135"/>
-      <c r="I4" s="135"/>
-      <c r="J4" s="135"/>
-      <c r="K4" s="136"/>
-      <c r="L4" s="117"/>
-      <c r="M4" s="118"/>
-      <c r="N4" s="118"/>
-      <c r="O4" s="118"/>
-      <c r="P4" s="119"/>
-      <c r="Q4" s="126"/>
-      <c r="R4" s="127"/>
-      <c r="S4" s="127"/>
-      <c r="T4" s="128"/>
+      <c r="D4" s="115"/>
+      <c r="E4" s="116"/>
+      <c r="F4" s="117"/>
+      <c r="G4" s="109"/>
+      <c r="H4" s="110"/>
+      <c r="I4" s="110"/>
+      <c r="J4" s="110"/>
+      <c r="K4" s="111"/>
+      <c r="L4" s="140"/>
+      <c r="M4" s="141"/>
+      <c r="N4" s="141"/>
+      <c r="O4" s="141"/>
+      <c r="P4" s="142"/>
+      <c r="Q4" s="98"/>
+      <c r="R4" s="99"/>
+      <c r="S4" s="99"/>
+      <c r="T4" s="100"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="130"/>
+      <c r="A5" s="105"/>
       <c r="B5" s="91"/>
       <c r="C5" s="67"/>
       <c r="D5" s="23">
@@ -9761,192 +9764,183 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="96" t="s">
+      <c r="D65" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="99" t="s">
+      <c r="E65" s="125" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="93" t="s">
+      <c r="G65" s="119" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="108" t="s">
+      <c r="H65" s="131" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="108" t="s">
+      <c r="I65" s="131" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="93" t="s">
+      <c r="J65" s="119" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="102" t="s">
+      <c r="L65" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="105" t="s">
+      <c r="M65" s="128" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="105" t="s">
+      <c r="N65" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="102" t="s">
+      <c r="O65" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="111" t="s">
+      <c r="Q65" s="134" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="111" t="s">
+      <c r="R65" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="111" t="s">
+      <c r="S65" s="134" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="97"/>
-      <c r="E66" s="100"/>
-      <c r="G66" s="94"/>
-      <c r="H66" s="109"/>
-      <c r="I66" s="109"/>
-      <c r="J66" s="94"/>
-      <c r="L66" s="103"/>
-      <c r="M66" s="106"/>
-      <c r="N66" s="106"/>
-      <c r="O66" s="103"/>
-      <c r="Q66" s="112"/>
-      <c r="R66" s="112"/>
-      <c r="S66" s="112"/>
+      <c r="D66" s="123"/>
+      <c r="E66" s="126"/>
+      <c r="G66" s="120"/>
+      <c r="H66" s="132"/>
+      <c r="I66" s="132"/>
+      <c r="J66" s="120"/>
+      <c r="L66" s="102"/>
+      <c r="M66" s="129"/>
+      <c r="N66" s="129"/>
+      <c r="O66" s="102"/>
+      <c r="Q66" s="135"/>
+      <c r="R66" s="135"/>
+      <c r="S66" s="135"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="97"/>
-      <c r="E67" s="100"/>
-      <c r="G67" s="94"/>
-      <c r="H67" s="109"/>
-      <c r="I67" s="109"/>
-      <c r="J67" s="94"/>
-      <c r="L67" s="103"/>
-      <c r="M67" s="106"/>
-      <c r="N67" s="106"/>
-      <c r="O67" s="103"/>
-      <c r="Q67" s="112"/>
-      <c r="R67" s="112"/>
-      <c r="S67" s="112"/>
+      <c r="D67" s="123"/>
+      <c r="E67" s="126"/>
+      <c r="G67" s="120"/>
+      <c r="H67" s="132"/>
+      <c r="I67" s="132"/>
+      <c r="J67" s="120"/>
+      <c r="L67" s="102"/>
+      <c r="M67" s="129"/>
+      <c r="N67" s="129"/>
+      <c r="O67" s="102"/>
+      <c r="Q67" s="135"/>
+      <c r="R67" s="135"/>
+      <c r="S67" s="135"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="97"/>
-      <c r="E68" s="100"/>
-      <c r="G68" s="94"/>
-      <c r="H68" s="109"/>
-      <c r="I68" s="109"/>
-      <c r="J68" s="94"/>
-      <c r="L68" s="103"/>
-      <c r="M68" s="106"/>
-      <c r="N68" s="106"/>
-      <c r="O68" s="103"/>
-      <c r="Q68" s="112"/>
-      <c r="R68" s="112"/>
-      <c r="S68" s="112"/>
+      <c r="D68" s="123"/>
+      <c r="E68" s="126"/>
+      <c r="G68" s="120"/>
+      <c r="H68" s="132"/>
+      <c r="I68" s="132"/>
+      <c r="J68" s="120"/>
+      <c r="L68" s="102"/>
+      <c r="M68" s="129"/>
+      <c r="N68" s="129"/>
+      <c r="O68" s="102"/>
+      <c r="Q68" s="135"/>
+      <c r="R68" s="135"/>
+      <c r="S68" s="135"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="97"/>
-      <c r="E69" s="100"/>
-      <c r="G69" s="94"/>
-      <c r="H69" s="109"/>
-      <c r="I69" s="109"/>
-      <c r="J69" s="94"/>
-      <c r="L69" s="103"/>
-      <c r="M69" s="106"/>
-      <c r="N69" s="106"/>
-      <c r="O69" s="103"/>
-      <c r="Q69" s="112"/>
-      <c r="R69" s="112"/>
-      <c r="S69" s="112"/>
+      <c r="D69" s="123"/>
+      <c r="E69" s="126"/>
+      <c r="G69" s="120"/>
+      <c r="H69" s="132"/>
+      <c r="I69" s="132"/>
+      <c r="J69" s="120"/>
+      <c r="L69" s="102"/>
+      <c r="M69" s="129"/>
+      <c r="N69" s="129"/>
+      <c r="O69" s="102"/>
+      <c r="Q69" s="135"/>
+      <c r="R69" s="135"/>
+      <c r="S69" s="135"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="97"/>
-      <c r="E70" s="100"/>
-      <c r="G70" s="94"/>
-      <c r="H70" s="109"/>
-      <c r="I70" s="109"/>
-      <c r="J70" s="94"/>
-      <c r="L70" s="103"/>
-      <c r="M70" s="106"/>
-      <c r="N70" s="106"/>
-      <c r="O70" s="103"/>
-      <c r="Q70" s="112"/>
-      <c r="R70" s="112"/>
-      <c r="S70" s="112"/>
+      <c r="D70" s="123"/>
+      <c r="E70" s="126"/>
+      <c r="G70" s="120"/>
+      <c r="H70" s="132"/>
+      <c r="I70" s="132"/>
+      <c r="J70" s="120"/>
+      <c r="L70" s="102"/>
+      <c r="M70" s="129"/>
+      <c r="N70" s="129"/>
+      <c r="O70" s="102"/>
+      <c r="Q70" s="135"/>
+      <c r="R70" s="135"/>
+      <c r="S70" s="135"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="97"/>
-      <c r="E71" s="100"/>
-      <c r="G71" s="94"/>
-      <c r="H71" s="109"/>
-      <c r="I71" s="109"/>
-      <c r="J71" s="94"/>
-      <c r="L71" s="103"/>
-      <c r="M71" s="106"/>
-      <c r="N71" s="106"/>
-      <c r="O71" s="103"/>
-      <c r="Q71" s="112"/>
-      <c r="R71" s="112"/>
-      <c r="S71" s="112"/>
+      <c r="D71" s="123"/>
+      <c r="E71" s="126"/>
+      <c r="G71" s="120"/>
+      <c r="H71" s="132"/>
+      <c r="I71" s="132"/>
+      <c r="J71" s="120"/>
+      <c r="L71" s="102"/>
+      <c r="M71" s="129"/>
+      <c r="N71" s="129"/>
+      <c r="O71" s="102"/>
+      <c r="Q71" s="135"/>
+      <c r="R71" s="135"/>
+      <c r="S71" s="135"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="97"/>
-      <c r="E72" s="100"/>
-      <c r="G72" s="94"/>
-      <c r="H72" s="109"/>
-      <c r="I72" s="109"/>
-      <c r="J72" s="94"/>
-      <c r="L72" s="103"/>
-      <c r="M72" s="106"/>
-      <c r="N72" s="106"/>
-      <c r="O72" s="103"/>
-      <c r="Q72" s="112"/>
-      <c r="R72" s="112"/>
-      <c r="S72" s="112"/>
+      <c r="D72" s="123"/>
+      <c r="E72" s="126"/>
+      <c r="G72" s="120"/>
+      <c r="H72" s="132"/>
+      <c r="I72" s="132"/>
+      <c r="J72" s="120"/>
+      <c r="L72" s="102"/>
+      <c r="M72" s="129"/>
+      <c r="N72" s="129"/>
+      <c r="O72" s="102"/>
+      <c r="Q72" s="135"/>
+      <c r="R72" s="135"/>
+      <c r="S72" s="135"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="97"/>
-      <c r="E73" s="100"/>
-      <c r="G73" s="94"/>
-      <c r="H73" s="109"/>
-      <c r="I73" s="109"/>
-      <c r="J73" s="94"/>
-      <c r="L73" s="103"/>
-      <c r="M73" s="106"/>
-      <c r="N73" s="106"/>
-      <c r="O73" s="103"/>
-      <c r="Q73" s="112"/>
-      <c r="R73" s="112"/>
-      <c r="S73" s="112"/>
+      <c r="D73" s="123"/>
+      <c r="E73" s="126"/>
+      <c r="G73" s="120"/>
+      <c r="H73" s="132"/>
+      <c r="I73" s="132"/>
+      <c r="J73" s="120"/>
+      <c r="L73" s="102"/>
+      <c r="M73" s="129"/>
+      <c r="N73" s="129"/>
+      <c r="O73" s="102"/>
+      <c r="Q73" s="135"/>
+      <c r="R73" s="135"/>
+      <c r="S73" s="135"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="98"/>
-      <c r="E74" s="101"/>
-      <c r="G74" s="95"/>
-      <c r="H74" s="110"/>
-      <c r="I74" s="110"/>
-      <c r="J74" s="95"/>
-      <c r="L74" s="104"/>
-      <c r="M74" s="107"/>
-      <c r="N74" s="107"/>
-      <c r="O74" s="104"/>
-      <c r="Q74" s="113"/>
-      <c r="R74" s="113"/>
-      <c r="S74" s="113"/>
+      <c r="D74" s="124"/>
+      <c r="E74" s="127"/>
+      <c r="G74" s="121"/>
+      <c r="H74" s="133"/>
+      <c r="I74" s="133"/>
+      <c r="J74" s="121"/>
+      <c r="L74" s="103"/>
+      <c r="M74" s="130"/>
+      <c r="N74" s="130"/>
+      <c r="O74" s="103"/>
+      <c r="Q74" s="136"/>
+      <c r="R74" s="136"/>
+      <c r="S74" s="136"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9963,6 +9957,15 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
corregí la pregunta 76
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5459A84D-E359-408E-A240-65C83EEF8EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F50D0F-E61B-4C8C-8FFA-BBE5CE2FD278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -983,7 +983,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1053,12 +1053,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1277,7 +1271,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1546,6 +1540,90 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1573,15 +1651,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1624,82 +1693,8 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -2773,7 +2768,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B23" s="144" t="s">
+      <c r="B23" s="53" t="s">
         <v>167</v>
       </c>
       <c r="C23" s="50" t="s">
@@ -2800,7 +2795,7 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B24" s="144" t="s">
+      <c r="B24" s="53" t="s">
         <v>199</v>
       </c>
       <c r="C24" s="50" t="s">
@@ -2827,7 +2822,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B25" s="144" t="s">
+      <c r="B25" s="53" t="s">
         <v>69</v>
       </c>
       <c r="C25" s="50" t="s">
@@ -2854,7 +2849,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="B26" s="144" t="s">
+      <c r="B26" s="53" t="s">
         <v>241</v>
       </c>
       <c r="C26" s="50" t="s">
@@ -2881,7 +2876,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="B27" s="144" t="s">
+      <c r="B27" s="53" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="50" t="s">
@@ -2908,7 +2903,7 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="B28" s="144" t="s">
+      <c r="B28" s="53" t="s">
         <v>77</v>
       </c>
       <c r="C28" s="50" t="s">
@@ -2935,7 +2930,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B29" s="144" t="s">
+      <c r="B29" s="53" t="s">
         <v>246</v>
       </c>
       <c r="C29" s="50" t="s">
@@ -2962,7 +2957,7 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="B30" s="143" t="s">
+      <c r="B30" s="145" t="s">
         <v>223</v>
       </c>
       <c r="C30" s="50" t="s">
@@ -2989,7 +2984,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B31" s="143" t="s">
+      <c r="B31" s="145" t="s">
         <v>207</v>
       </c>
       <c r="C31" s="50" t="s">
@@ -3016,7 +3011,7 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="B32" s="143" t="s">
+      <c r="B32" s="145" t="s">
         <v>211</v>
       </c>
       <c r="C32" s="50" t="s">
@@ -3043,7 +3038,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B33" s="143" t="s">
+      <c r="B33" s="145" t="s">
         <v>215</v>
       </c>
       <c r="C33" s="50" t="s">
@@ -3070,7 +3065,7 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="B34" s="143" t="s">
+      <c r="B34" s="145" t="s">
         <v>227</v>
       </c>
       <c r="C34" s="50" t="s">
@@ -3097,7 +3092,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B35" s="143" t="s">
+      <c r="B35" s="145" t="s">
         <v>73</v>
       </c>
       <c r="C35" s="50" t="s">
@@ -3124,7 +3119,7 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="B36" s="50" t="s">
+      <c r="B36" s="143" t="s">
         <v>129</v>
       </c>
       <c r="C36" s="50" t="s">
@@ -3151,7 +3146,7 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="B37" s="50" t="s">
+      <c r="B37" s="144" t="s">
         <v>82</v>
       </c>
       <c r="C37" s="50" t="s">
@@ -3178,7 +3173,7 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="B38" s="50" t="s">
+      <c r="B38" s="143" t="s">
         <v>37</v>
       </c>
       <c r="C38" s="50" t="s">
@@ -3205,7 +3200,7 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="B39" s="50" t="s">
+      <c r="B39" s="143" t="s">
         <v>60</v>
       </c>
       <c r="C39" s="50" t="s">
@@ -3232,7 +3227,7 @@
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="B40" s="50" t="s">
+      <c r="B40" s="143" t="s">
         <v>181</v>
       </c>
       <c r="C40" s="50" t="s">
@@ -3259,7 +3254,7 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="B41" s="50" t="s">
+      <c r="B41" s="143" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="50" t="s">
@@ -3286,7 +3281,7 @@
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="B42" s="50" t="s">
+      <c r="B42" s="143" t="s">
         <v>143</v>
       </c>
       <c r="C42" s="50" t="s">
@@ -7116,30 +7111,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="118" t="s">
+      <c r="B1" s="92" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
-      <c r="P1" s="118"/>
-      <c r="Q1" s="118"/>
-      <c r="R1" s="118"/>
-      <c r="S1" s="118"/>
-      <c r="T1" s="118"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+      <c r="I1" s="92"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="92"/>
+      <c r="O1" s="92"/>
+      <c r="P1" s="92"/>
+      <c r="Q1" s="92"/>
+      <c r="R1" s="92"/>
+      <c r="S1" s="92"/>
+      <c r="T1" s="92"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="129" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="90" t="s">
@@ -7148,89 +7143,89 @@
       <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="92" t="str">
+      <c r="D2" s="120" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="93"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="92" t="str">
+      <c r="E2" s="121"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="120" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
-      <c r="J2" s="93"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="92" t="s">
+      <c r="H2" s="121"/>
+      <c r="I2" s="121"/>
+      <c r="J2" s="121"/>
+      <c r="K2" s="122"/>
+      <c r="L2" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="93"/>
-      <c r="N2" s="93"/>
-      <c r="O2" s="93"/>
-      <c r="P2" s="94"/>
-      <c r="Q2" s="92" t="str">
+      <c r="M2" s="121"/>
+      <c r="N2" s="121"/>
+      <c r="O2" s="121"/>
+      <c r="P2" s="122"/>
+      <c r="Q2" s="120" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="93"/>
-      <c r="S2" s="93"/>
-      <c r="T2" s="94"/>
+      <c r="R2" s="121"/>
+      <c r="S2" s="121"/>
+      <c r="T2" s="122"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="105"/>
+      <c r="A3" s="130"/>
       <c r="B3" s="91"/>
       <c r="C3" s="67"/>
-      <c r="D3" s="112" t="s">
+      <c r="D3" s="137" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="113"/>
-      <c r="F3" s="114"/>
-      <c r="G3" s="106" t="s">
+      <c r="E3" s="138"/>
+      <c r="F3" s="139"/>
+      <c r="G3" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="107"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="137" t="s">
+      <c r="H3" s="132"/>
+      <c r="I3" s="132"/>
+      <c r="J3" s="132"/>
+      <c r="K3" s="133"/>
+      <c r="L3" s="114" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="138"/>
-      <c r="N3" s="138"/>
-      <c r="O3" s="138"/>
-      <c r="P3" s="139"/>
-      <c r="Q3" s="95" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="96"/>
-      <c r="S3" s="96"/>
-      <c r="T3" s="97"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="116"/>
+      <c r="Q3" s="123" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="124"/>
+      <c r="S3" s="124"/>
+      <c r="T3" s="125"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="105"/>
+      <c r="A4" s="130"/>
       <c r="B4" s="91"/>
       <c r="C4" s="67"/>
-      <c r="D4" s="115"/>
-      <c r="E4" s="116"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="109"/>
-      <c r="H4" s="110"/>
-      <c r="I4" s="110"/>
-      <c r="J4" s="110"/>
-      <c r="K4" s="111"/>
-      <c r="L4" s="140"/>
-      <c r="M4" s="141"/>
-      <c r="N4" s="141"/>
-      <c r="O4" s="141"/>
-      <c r="P4" s="142"/>
-      <c r="Q4" s="98"/>
-      <c r="R4" s="99"/>
-      <c r="S4" s="99"/>
-      <c r="T4" s="100"/>
+      <c r="D4" s="140"/>
+      <c r="E4" s="141"/>
+      <c r="F4" s="142"/>
+      <c r="G4" s="134"/>
+      <c r="H4" s="135"/>
+      <c r="I4" s="135"/>
+      <c r="J4" s="135"/>
+      <c r="K4" s="136"/>
+      <c r="L4" s="117"/>
+      <c r="M4" s="118"/>
+      <c r="N4" s="118"/>
+      <c r="O4" s="118"/>
+      <c r="P4" s="119"/>
+      <c r="Q4" s="126"/>
+      <c r="R4" s="127"/>
+      <c r="S4" s="127"/>
+      <c r="T4" s="128"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="105"/>
+      <c r="A5" s="130"/>
       <c r="B5" s="91"/>
       <c r="C5" s="67"/>
       <c r="D5" s="23">
@@ -9764,183 +9759,192 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="122" t="s">
+      <c r="D65" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="125" t="s">
+      <c r="E65" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="119" t="s">
+      <c r="G65" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="131" t="s">
+      <c r="H65" s="108" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="131" t="s">
+      <c r="I65" s="108" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="119" t="s">
+      <c r="J65" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="101" t="s">
+      <c r="L65" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="128" t="s">
+      <c r="M65" s="105" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="128" t="s">
+      <c r="N65" s="105" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="101" t="s">
+      <c r="O65" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="134" t="s">
+      <c r="Q65" s="111" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="134" t="s">
+      <c r="R65" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="134" t="s">
+      <c r="S65" s="111" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="123"/>
-      <c r="E66" s="126"/>
-      <c r="G66" s="120"/>
-      <c r="H66" s="132"/>
-      <c r="I66" s="132"/>
-      <c r="J66" s="120"/>
-      <c r="L66" s="102"/>
-      <c r="M66" s="129"/>
-      <c r="N66" s="129"/>
-      <c r="O66" s="102"/>
-      <c r="Q66" s="135"/>
-      <c r="R66" s="135"/>
-      <c r="S66" s="135"/>
+      <c r="D66" s="97"/>
+      <c r="E66" s="100"/>
+      <c r="G66" s="94"/>
+      <c r="H66" s="109"/>
+      <c r="I66" s="109"/>
+      <c r="J66" s="94"/>
+      <c r="L66" s="103"/>
+      <c r="M66" s="106"/>
+      <c r="N66" s="106"/>
+      <c r="O66" s="103"/>
+      <c r="Q66" s="112"/>
+      <c r="R66" s="112"/>
+      <c r="S66" s="112"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="123"/>
-      <c r="E67" s="126"/>
-      <c r="G67" s="120"/>
-      <c r="H67" s="132"/>
-      <c r="I67" s="132"/>
-      <c r="J67" s="120"/>
-      <c r="L67" s="102"/>
-      <c r="M67" s="129"/>
-      <c r="N67" s="129"/>
-      <c r="O67" s="102"/>
-      <c r="Q67" s="135"/>
-      <c r="R67" s="135"/>
-      <c r="S67" s="135"/>
+      <c r="D67" s="97"/>
+      <c r="E67" s="100"/>
+      <c r="G67" s="94"/>
+      <c r="H67" s="109"/>
+      <c r="I67" s="109"/>
+      <c r="J67" s="94"/>
+      <c r="L67" s="103"/>
+      <c r="M67" s="106"/>
+      <c r="N67" s="106"/>
+      <c r="O67" s="103"/>
+      <c r="Q67" s="112"/>
+      <c r="R67" s="112"/>
+      <c r="S67" s="112"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="123"/>
-      <c r="E68" s="126"/>
-      <c r="G68" s="120"/>
-      <c r="H68" s="132"/>
-      <c r="I68" s="132"/>
-      <c r="J68" s="120"/>
-      <c r="L68" s="102"/>
-      <c r="M68" s="129"/>
-      <c r="N68" s="129"/>
-      <c r="O68" s="102"/>
-      <c r="Q68" s="135"/>
-      <c r="R68" s="135"/>
-      <c r="S68" s="135"/>
+      <c r="D68" s="97"/>
+      <c r="E68" s="100"/>
+      <c r="G68" s="94"/>
+      <c r="H68" s="109"/>
+      <c r="I68" s="109"/>
+      <c r="J68" s="94"/>
+      <c r="L68" s="103"/>
+      <c r="M68" s="106"/>
+      <c r="N68" s="106"/>
+      <c r="O68" s="103"/>
+      <c r="Q68" s="112"/>
+      <c r="R68" s="112"/>
+      <c r="S68" s="112"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="123"/>
-      <c r="E69" s="126"/>
-      <c r="G69" s="120"/>
-      <c r="H69" s="132"/>
-      <c r="I69" s="132"/>
-      <c r="J69" s="120"/>
-      <c r="L69" s="102"/>
-      <c r="M69" s="129"/>
-      <c r="N69" s="129"/>
-      <c r="O69" s="102"/>
-      <c r="Q69" s="135"/>
-      <c r="R69" s="135"/>
-      <c r="S69" s="135"/>
+      <c r="D69" s="97"/>
+      <c r="E69" s="100"/>
+      <c r="G69" s="94"/>
+      <c r="H69" s="109"/>
+      <c r="I69" s="109"/>
+      <c r="J69" s="94"/>
+      <c r="L69" s="103"/>
+      <c r="M69" s="106"/>
+      <c r="N69" s="106"/>
+      <c r="O69" s="103"/>
+      <c r="Q69" s="112"/>
+      <c r="R69" s="112"/>
+      <c r="S69" s="112"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="123"/>
-      <c r="E70" s="126"/>
-      <c r="G70" s="120"/>
-      <c r="H70" s="132"/>
-      <c r="I70" s="132"/>
-      <c r="J70" s="120"/>
-      <c r="L70" s="102"/>
-      <c r="M70" s="129"/>
-      <c r="N70" s="129"/>
-      <c r="O70" s="102"/>
-      <c r="Q70" s="135"/>
-      <c r="R70" s="135"/>
-      <c r="S70" s="135"/>
+      <c r="D70" s="97"/>
+      <c r="E70" s="100"/>
+      <c r="G70" s="94"/>
+      <c r="H70" s="109"/>
+      <c r="I70" s="109"/>
+      <c r="J70" s="94"/>
+      <c r="L70" s="103"/>
+      <c r="M70" s="106"/>
+      <c r="N70" s="106"/>
+      <c r="O70" s="103"/>
+      <c r="Q70" s="112"/>
+      <c r="R70" s="112"/>
+      <c r="S70" s="112"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="123"/>
-      <c r="E71" s="126"/>
-      <c r="G71" s="120"/>
-      <c r="H71" s="132"/>
-      <c r="I71" s="132"/>
-      <c r="J71" s="120"/>
-      <c r="L71" s="102"/>
-      <c r="M71" s="129"/>
-      <c r="N71" s="129"/>
-      <c r="O71" s="102"/>
-      <c r="Q71" s="135"/>
-      <c r="R71" s="135"/>
-      <c r="S71" s="135"/>
+      <c r="D71" s="97"/>
+      <c r="E71" s="100"/>
+      <c r="G71" s="94"/>
+      <c r="H71" s="109"/>
+      <c r="I71" s="109"/>
+      <c r="J71" s="94"/>
+      <c r="L71" s="103"/>
+      <c r="M71" s="106"/>
+      <c r="N71" s="106"/>
+      <c r="O71" s="103"/>
+      <c r="Q71" s="112"/>
+      <c r="R71" s="112"/>
+      <c r="S71" s="112"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="123"/>
-      <c r="E72" s="126"/>
-      <c r="G72" s="120"/>
-      <c r="H72" s="132"/>
-      <c r="I72" s="132"/>
-      <c r="J72" s="120"/>
-      <c r="L72" s="102"/>
-      <c r="M72" s="129"/>
-      <c r="N72" s="129"/>
-      <c r="O72" s="102"/>
-      <c r="Q72" s="135"/>
-      <c r="R72" s="135"/>
-      <c r="S72" s="135"/>
+      <c r="D72" s="97"/>
+      <c r="E72" s="100"/>
+      <c r="G72" s="94"/>
+      <c r="H72" s="109"/>
+      <c r="I72" s="109"/>
+      <c r="J72" s="94"/>
+      <c r="L72" s="103"/>
+      <c r="M72" s="106"/>
+      <c r="N72" s="106"/>
+      <c r="O72" s="103"/>
+      <c r="Q72" s="112"/>
+      <c r="R72" s="112"/>
+      <c r="S72" s="112"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="123"/>
-      <c r="E73" s="126"/>
-      <c r="G73" s="120"/>
-      <c r="H73" s="132"/>
-      <c r="I73" s="132"/>
-      <c r="J73" s="120"/>
-      <c r="L73" s="102"/>
-      <c r="M73" s="129"/>
-      <c r="N73" s="129"/>
-      <c r="O73" s="102"/>
-      <c r="Q73" s="135"/>
-      <c r="R73" s="135"/>
-      <c r="S73" s="135"/>
+      <c r="D73" s="97"/>
+      <c r="E73" s="100"/>
+      <c r="G73" s="94"/>
+      <c r="H73" s="109"/>
+      <c r="I73" s="109"/>
+      <c r="J73" s="94"/>
+      <c r="L73" s="103"/>
+      <c r="M73" s="106"/>
+      <c r="N73" s="106"/>
+      <c r="O73" s="103"/>
+      <c r="Q73" s="112"/>
+      <c r="R73" s="112"/>
+      <c r="S73" s="112"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="124"/>
-      <c r="E74" s="127"/>
-      <c r="G74" s="121"/>
-      <c r="H74" s="133"/>
-      <c r="I74" s="133"/>
-      <c r="J74" s="121"/>
-      <c r="L74" s="103"/>
-      <c r="M74" s="130"/>
-      <c r="N74" s="130"/>
-      <c r="O74" s="103"/>
-      <c r="Q74" s="136"/>
-      <c r="R74" s="136"/>
-      <c r="S74" s="136"/>
+      <c r="D74" s="98"/>
+      <c r="E74" s="101"/>
+      <c r="G74" s="95"/>
+      <c r="H74" s="110"/>
+      <c r="I74" s="110"/>
+      <c r="J74" s="95"/>
+      <c r="L74" s="104"/>
+      <c r="M74" s="107"/>
+      <c r="N74" s="107"/>
+      <c r="O74" s="104"/>
+      <c r="Q74" s="113"/>
+      <c r="R74" s="113"/>
+      <c r="S74" s="113"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9957,15 +9961,6 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
clase de hoy es sobre el módulo 7 y 8
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F50D0F-E61B-4C8C-8FFA-BBE5CE2FD278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67C029E-DC16-418A-84F8-FD7F2DDFA3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -217,9 +217,6 @@
     <t>3135975782</t>
   </si>
   <si>
-    <t>GABRIELABARRETOH1211@GMAIL.COM</t>
-  </si>
-  <si>
     <t xml:space="preserve">PLUTARCO DAVID SAENZ URANGO </t>
   </si>
   <si>
@@ -806,6 +803,9 @@
   </si>
   <si>
     <t>IE JOSÉ MARÍA CÓRDOBA</t>
+  </si>
+  <si>
+    <t>GABRIELABARRETOH1211@GMAIL.COM, gabrielabarretoh1211@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1271,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1426,6 +1426,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1540,6 +1542,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1570,15 +1650,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1624,78 +1695,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -2202,28 +2201,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="57"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -2256,25 +2255,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C4" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D4" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="50" t="s">
         <v>92</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="F4" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="F4" s="51" t="s">
+      <c r="G4" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="G4" s="50" t="s">
-        <v>95</v>
-      </c>
       <c r="H4" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2283,25 +2282,25 @@
         <v>2</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C5" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D5" s="51" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="50" t="s">
         <v>149</v>
       </c>
-      <c r="E5" s="50" t="s">
+      <c r="F5" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="F5" s="51" t="s">
+      <c r="G5" s="50" t="s">
         <v>151</v>
       </c>
-      <c r="G5" s="50" t="s">
-        <v>152</v>
-      </c>
       <c r="H5" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2310,25 +2309,25 @@
         <v>3</v>
       </c>
       <c r="B6" s="50" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D6" s="51" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E6" s="50" t="s">
         <v>57</v>
       </c>
       <c r="F6" s="51" t="s">
+        <v>204</v>
+      </c>
+      <c r="G6" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="G6" s="50" t="s">
-        <v>206</v>
-      </c>
       <c r="H6" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2337,25 +2336,25 @@
         <v>4</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>30</v>
       </c>
       <c r="D7" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7" s="50" t="s">
         <v>154</v>
       </c>
-      <c r="E7" s="50" t="s">
+      <c r="F7" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="F7" s="51" t="s">
+      <c r="G7" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="G7" s="50" t="s">
-        <v>157</v>
-      </c>
       <c r="H7" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2364,25 +2363,25 @@
         <v>5</v>
       </c>
       <c r="B8" s="50" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D8" s="51" t="s">
+        <v>195</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" s="51" t="s">
         <v>196</v>
       </c>
-      <c r="E8" s="50" t="s">
-        <v>192</v>
-      </c>
-      <c r="F8" s="51" t="s">
+      <c r="G8" s="50" t="s">
         <v>197</v>
       </c>
-      <c r="G8" s="50" t="s">
-        <v>198</v>
-      </c>
       <c r="H8" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2391,25 +2390,25 @@
         <v>6</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C9" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D9" s="51" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" s="50" t="s">
         <v>177</v>
       </c>
-      <c r="E9" s="50" t="s">
+      <c r="F9" s="51" t="s">
         <v>178</v>
       </c>
-      <c r="F9" s="51" t="s">
+      <c r="G9" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="G9" s="50" t="s">
-        <v>180</v>
-      </c>
       <c r="H9" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2418,25 +2417,25 @@
         <v>7</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="50" t="s">
+      <c r="F10" s="51" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="51" t="s">
+      <c r="G10" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="G10" s="50" t="s">
-        <v>68</v>
-      </c>
       <c r="H10" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2445,25 +2444,25 @@
         <v>8</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C11" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D11" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="F11" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="E11" s="50" t="s">
-        <v>155</v>
-      </c>
-      <c r="F11" s="51" t="s">
+      <c r="G11" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="G11" s="50" t="s">
-        <v>161</v>
-      </c>
       <c r="H11" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2472,25 +2471,25 @@
         <v>9</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C12" s="50" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="51" t="s">
+        <v>236</v>
+      </c>
+      <c r="E12" s="50" t="s">
         <v>237</v>
       </c>
-      <c r="E12" s="50" t="s">
+      <c r="F12" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="F12" s="51" t="s">
+      <c r="G12" s="50" t="s">
         <v>239</v>
       </c>
-      <c r="G12" s="50" t="s">
-        <v>240</v>
-      </c>
       <c r="H12" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2499,25 +2498,25 @@
         <v>10</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C13" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D13" s="51" t="s">
+        <v>186</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="F13" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="E13" s="50" t="s">
-        <v>183</v>
-      </c>
-      <c r="F13" s="51" t="s">
+      <c r="G13" s="50" t="s">
         <v>188</v>
       </c>
-      <c r="G13" s="50" t="s">
-        <v>189</v>
-      </c>
       <c r="H13" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2526,25 +2525,25 @@
         <v>11</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C14" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D14" s="51" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="50" t="s">
         <v>139</v>
       </c>
-      <c r="E14" s="50" t="s">
+      <c r="F14" s="51" t="s">
         <v>140</v>
       </c>
-      <c r="F14" s="51" t="s">
+      <c r="G14" s="50" t="s">
         <v>141</v>
       </c>
-      <c r="G14" s="50" t="s">
-        <v>142</v>
-      </c>
       <c r="H14" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2553,25 +2552,25 @@
         <v>12</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D15" s="51" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="50" t="s">
         <v>101</v>
       </c>
-      <c r="E15" s="50" t="s">
+      <c r="F15" s="51" t="s">
         <v>102</v>
       </c>
-      <c r="F15" s="51" t="s">
+      <c r="G15" s="50" t="s">
         <v>103</v>
       </c>
-      <c r="G15" s="50" t="s">
-        <v>104</v>
-      </c>
       <c r="H15" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2580,25 +2579,25 @@
         <v>13</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D16" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="50" t="s">
+      <c r="F16" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="F16" s="51" t="s">
+      <c r="G16" s="50" t="s">
         <v>89</v>
       </c>
-      <c r="G16" s="50" t="s">
-        <v>90</v>
-      </c>
       <c r="H16" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2607,25 +2606,25 @@
         <v>14</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C17" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D17" s="51" t="s">
+        <v>219</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F17" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="E17" s="50" t="s">
-        <v>66</v>
-      </c>
-      <c r="F17" s="51" t="s">
+      <c r="G17" s="50" t="s">
         <v>221</v>
       </c>
-      <c r="G17" s="50" t="s">
-        <v>222</v>
-      </c>
       <c r="H17" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2634,25 +2633,25 @@
         <v>15</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D18" s="51" t="s">
+        <v>251</v>
+      </c>
+      <c r="E18" s="50" t="s">
+        <v>247</v>
+      </c>
+      <c r="F18" s="51" t="s">
         <v>252</v>
       </c>
-      <c r="E18" s="50" t="s">
-        <v>248</v>
-      </c>
-      <c r="F18" s="51" t="s">
+      <c r="G18" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="G18" s="50" t="s">
+      <c r="H18" s="50" t="s">
         <v>254</v>
-      </c>
-      <c r="H18" s="50" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2679,7 +2678,7 @@
         <v>36</v>
       </c>
       <c r="H19" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2703,10 +2702,10 @@
         <v>58</v>
       </c>
       <c r="G20" s="50" t="s">
-        <v>59</v>
+        <v>255</v>
       </c>
       <c r="H20" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2715,25 +2714,25 @@
         <v>18</v>
       </c>
       <c r="B21" s="53" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C21" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D21" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="E21" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="50" t="s">
+      <c r="F21" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="F21" s="51" t="s">
+      <c r="G21" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="G21" s="50" t="s">
-        <v>118</v>
-      </c>
       <c r="H21" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2742,25 +2741,25 @@
         <v>19</v>
       </c>
       <c r="B22" s="53" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C22" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D22" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="E22" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="E22" s="50" t="s">
+      <c r="F22" s="51" t="s">
         <v>126</v>
       </c>
-      <c r="F22" s="51" t="s">
+      <c r="G22" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="G22" s="50" t="s">
-        <v>128</v>
-      </c>
       <c r="H22" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2769,25 +2768,25 @@
         <v>20</v>
       </c>
       <c r="B23" s="53" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C23" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D23" s="51" t="s">
+        <v>167</v>
+      </c>
+      <c r="E23" s="50" t="s">
         <v>168</v>
       </c>
-      <c r="E23" s="50" t="s">
+      <c r="F23" s="51" t="s">
         <v>169</v>
       </c>
-      <c r="F23" s="51" t="s">
+      <c r="G23" s="50" t="s">
         <v>170</v>
       </c>
-      <c r="G23" s="50" t="s">
-        <v>171</v>
-      </c>
       <c r="H23" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2796,25 +2795,25 @@
         <v>21</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C24" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E24" s="50" t="s">
         <v>34</v>
       </c>
       <c r="F24" s="51" t="s">
+        <v>200</v>
+      </c>
+      <c r="G24" s="50" t="s">
         <v>201</v>
       </c>
-      <c r="G24" s="50" t="s">
-        <v>202</v>
-      </c>
       <c r="H24" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2823,25 +2822,25 @@
         <v>22</v>
       </c>
       <c r="B25" s="53" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C25" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D25" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="50" t="s">
-        <v>66</v>
-      </c>
-      <c r="F25" s="51" t="s">
+      <c r="G25" s="50" t="s">
         <v>71</v>
       </c>
-      <c r="G25" s="50" t="s">
-        <v>72</v>
-      </c>
       <c r="H25" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2850,25 +2849,25 @@
         <v>23</v>
       </c>
       <c r="B26" s="53" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C26" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D26" s="51" t="s">
+        <v>241</v>
+      </c>
+      <c r="E26" s="50" t="s">
         <v>242</v>
       </c>
-      <c r="E26" s="50" t="s">
+      <c r="F26" s="51" t="s">
         <v>243</v>
       </c>
-      <c r="F26" s="51" t="s">
+      <c r="G26" s="50" t="s">
         <v>244</v>
       </c>
-      <c r="G26" s="50" t="s">
-        <v>245</v>
-      </c>
       <c r="H26" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2895,7 +2894,7 @@
         <v>44</v>
       </c>
       <c r="H27" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2904,25 +2903,25 @@
         <v>25</v>
       </c>
       <c r="B28" s="53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D28" s="51" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="E28" s="50" t="s">
+      <c r="F28" s="51" t="s">
         <v>79</v>
       </c>
-      <c r="F28" s="51" t="s">
+      <c r="G28" s="50" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="50" t="s">
-        <v>81</v>
-      </c>
       <c r="H28" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2931,25 +2930,25 @@
         <v>26</v>
       </c>
       <c r="B29" s="53" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C29" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D29" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="E29" s="50" t="s">
         <v>247</v>
       </c>
-      <c r="E29" s="50" t="s">
+      <c r="F29" s="51" t="s">
         <v>248</v>
       </c>
-      <c r="F29" s="51" t="s">
+      <c r="G29" s="50" t="s">
         <v>249</v>
       </c>
-      <c r="G29" s="50" t="s">
-        <v>250</v>
-      </c>
       <c r="H29" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2957,26 +2956,26 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="B30" s="145" t="s">
-        <v>223</v>
+      <c r="B30" s="53" t="s">
+        <v>222</v>
       </c>
       <c r="C30" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D30" s="51" t="s">
+        <v>223</v>
+      </c>
+      <c r="E30" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" s="51" t="s">
         <v>224</v>
       </c>
-      <c r="E30" s="50" t="s">
-        <v>66</v>
-      </c>
-      <c r="F30" s="51" t="s">
+      <c r="G30" s="50" t="s">
         <v>225</v>
       </c>
-      <c r="G30" s="50" t="s">
-        <v>226</v>
-      </c>
       <c r="H30" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2984,26 +2983,26 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B31" s="145" t="s">
-        <v>207</v>
+      <c r="B31" s="53" t="s">
+        <v>206</v>
       </c>
       <c r="C31" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D31" s="51" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E31" s="50" t="s">
         <v>57</v>
       </c>
       <c r="F31" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="G31" s="50" t="s">
         <v>209</v>
       </c>
-      <c r="G31" s="50" t="s">
-        <v>210</v>
-      </c>
       <c r="H31" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3011,26 +3010,26 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="B32" s="145" t="s">
-        <v>211</v>
+      <c r="B32" s="53" t="s">
+        <v>210</v>
       </c>
       <c r="C32" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D32" s="51" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E32" s="50" t="s">
         <v>57</v>
       </c>
       <c r="F32" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="G32" s="50" t="s">
         <v>213</v>
       </c>
-      <c r="G32" s="50" t="s">
-        <v>214</v>
-      </c>
       <c r="H32" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3038,26 +3037,26 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B33" s="145" t="s">
-        <v>215</v>
+      <c r="B33" s="53" t="s">
+        <v>214</v>
       </c>
       <c r="C33" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E33" s="50" t="s">
         <v>57</v>
       </c>
       <c r="F33" s="51" t="s">
+        <v>216</v>
+      </c>
+      <c r="G33" s="50" t="s">
         <v>217</v>
       </c>
-      <c r="G33" s="50" t="s">
-        <v>218</v>
-      </c>
       <c r="H33" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3065,26 +3064,26 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="B34" s="145" t="s">
-        <v>227</v>
+      <c r="B34" s="53" t="s">
+        <v>226</v>
       </c>
       <c r="C34" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D34" s="51" t="s">
+        <v>227</v>
+      </c>
+      <c r="E34" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F34" s="51" t="s">
         <v>228</v>
       </c>
-      <c r="E34" s="50" t="s">
-        <v>66</v>
-      </c>
-      <c r="F34" s="51" t="s">
+      <c r="G34" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="G34" s="50" t="s">
-        <v>230</v>
-      </c>
       <c r="H34" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3092,26 +3091,26 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B35" s="145" t="s">
-        <v>73</v>
+      <c r="B35" s="53" t="s">
+        <v>72</v>
       </c>
       <c r="C35" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D35" s="51" t="s">
+        <v>73</v>
+      </c>
+      <c r="E35" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F35" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="E35" s="50" t="s">
-        <v>66</v>
-      </c>
-      <c r="F35" s="51" t="s">
+      <c r="G35" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="G35" s="50" t="s">
-        <v>76</v>
-      </c>
       <c r="H35" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3119,26 +3118,26 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="B36" s="143" t="s">
-        <v>129</v>
+      <c r="B36" s="54" t="s">
+        <v>128</v>
       </c>
       <c r="C36" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D36" s="51" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="50" t="s">
+      <c r="F36" s="51" t="s">
         <v>131</v>
       </c>
-      <c r="F36" s="51" t="s">
+      <c r="G36" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="G36" s="50" t="s">
-        <v>133</v>
-      </c>
       <c r="H36" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3146,26 +3145,26 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="B37" s="144" t="s">
-        <v>82</v>
+      <c r="B37" s="55" t="s">
+        <v>81</v>
       </c>
       <c r="C37" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D37" s="51" t="s">
+        <v>82</v>
+      </c>
+      <c r="E37" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="E37" s="50" t="s">
-        <v>79</v>
-      </c>
-      <c r="F37" s="51" t="s">
+      <c r="G37" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="G37" s="50" t="s">
-        <v>85</v>
-      </c>
       <c r="H37" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3173,7 +3172,7 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="B38" s="143" t="s">
+      <c r="B38" s="54" t="s">
         <v>37</v>
       </c>
       <c r="C38" s="50" t="s">
@@ -3192,7 +3191,7 @@
         <v>40</v>
       </c>
       <c r="H38" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3200,26 +3199,26 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="B39" s="143" t="s">
-        <v>60</v>
+      <c r="B39" s="54" t="s">
+        <v>59</v>
       </c>
       <c r="C39" s="50" t="s">
         <v>30</v>
       </c>
       <c r="D39" s="51" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E39" s="50" t="s">
         <v>57</v>
       </c>
       <c r="F39" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="G39" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="G39" s="50" t="s">
-        <v>63</v>
-      </c>
       <c r="H39" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3227,26 +3226,26 @@
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="B40" s="143" t="s">
-        <v>181</v>
+      <c r="B40" s="54" t="s">
+        <v>180</v>
       </c>
       <c r="C40" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D40" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="E40" s="50" t="s">
         <v>182</v>
       </c>
-      <c r="E40" s="50" t="s">
+      <c r="F40" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="F40" s="51" t="s">
+      <c r="G40" s="50" t="s">
         <v>184</v>
       </c>
-      <c r="G40" s="50" t="s">
-        <v>185</v>
-      </c>
       <c r="H40" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3254,7 +3253,7 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="B41" s="143" t="s">
+      <c r="B41" s="54" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="50" t="s">
@@ -3273,7 +3272,7 @@
         <v>54</v>
       </c>
       <c r="H41" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3281,26 +3280,26 @@
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="B42" s="143" t="s">
-        <v>143</v>
+      <c r="B42" s="54" t="s">
+        <v>142</v>
       </c>
       <c r="C42" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D42" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="E42" s="50" t="s">
         <v>144</v>
       </c>
-      <c r="E42" s="50" t="s">
+      <c r="F42" s="51" t="s">
         <v>145</v>
       </c>
-      <c r="F42" s="51" t="s">
+      <c r="G42" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="G42" s="50" t="s">
-        <v>147</v>
-      </c>
       <c r="H42" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3309,25 +3308,25 @@
         <v>40</v>
       </c>
       <c r="B43" s="50" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C43" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D43" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="E43" s="50" t="s">
+        <v>168</v>
+      </c>
+      <c r="F43" s="51" t="s">
         <v>173</v>
       </c>
-      <c r="E43" s="50" t="s">
-        <v>169</v>
-      </c>
-      <c r="F43" s="51" t="s">
+      <c r="G43" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="G43" s="50" t="s">
-        <v>175</v>
-      </c>
       <c r="H43" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3354,7 +3353,7 @@
         <v>49</v>
       </c>
       <c r="H44" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3363,25 +3362,25 @@
         <v>42</v>
       </c>
       <c r="B45" s="50" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C45" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D45" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="E45" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="E45" s="50" t="s">
+      <c r="F45" s="51" t="s">
         <v>121</v>
       </c>
-      <c r="F45" s="51" t="s">
+      <c r="G45" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="G45" s="50" t="s">
-        <v>123</v>
-      </c>
       <c r="H45" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3390,25 +3389,25 @@
         <v>43</v>
       </c>
       <c r="B46" s="50" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C46" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D46" s="51" t="s">
+        <v>96</v>
+      </c>
+      <c r="E46" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="F46" s="51" t="s">
         <v>97</v>
       </c>
-      <c r="E46" s="50" t="s">
-        <v>93</v>
-      </c>
-      <c r="F46" s="51" t="s">
+      <c r="G46" s="50" t="s">
         <v>98</v>
       </c>
-      <c r="G46" s="50" t="s">
-        <v>99</v>
-      </c>
       <c r="H46" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3417,25 +3416,25 @@
         <v>44</v>
       </c>
       <c r="B47" s="50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C47" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E47" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="E47" s="50" t="s">
+      <c r="F47" s="51" t="s">
         <v>164</v>
       </c>
-      <c r="F47" s="51" t="s">
+      <c r="G47" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="G47" s="50" t="s">
-        <v>166</v>
-      </c>
       <c r="H47" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3444,25 +3443,25 @@
         <v>45</v>
       </c>
       <c r="B48" s="50" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C48" s="50" t="s">
         <v>30</v>
       </c>
       <c r="D48" s="51" t="s">
+        <v>134</v>
+      </c>
+      <c r="E48" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="F48" s="51" t="s">
         <v>135</v>
       </c>
-      <c r="E48" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="F48" s="51" t="s">
+      <c r="G48" s="50" t="s">
         <v>136</v>
       </c>
-      <c r="G48" s="50" t="s">
-        <v>137</v>
-      </c>
       <c r="H48" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3471,25 +3470,25 @@
         <v>46</v>
       </c>
       <c r="B49" s="50" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C49" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="51" t="s">
+        <v>105</v>
+      </c>
+      <c r="E49" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="F49" s="51" t="s">
         <v>106</v>
       </c>
-      <c r="E49" s="50" t="s">
-        <v>102</v>
-      </c>
-      <c r="F49" s="51" t="s">
+      <c r="G49" s="50" t="s">
         <v>107</v>
       </c>
-      <c r="G49" s="50" t="s">
-        <v>108</v>
-      </c>
       <c r="H49" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3498,25 +3497,25 @@
         <v>47</v>
       </c>
       <c r="B50" s="50" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C50" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D50" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="E50" s="50" t="s">
         <v>232</v>
       </c>
-      <c r="E50" s="50" t="s">
+      <c r="F50" s="51" t="s">
         <v>233</v>
       </c>
-      <c r="F50" s="51" t="s">
+      <c r="G50" s="50" t="s">
         <v>234</v>
       </c>
-      <c r="G50" s="50" t="s">
-        <v>235</v>
-      </c>
       <c r="H50" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3525,25 +3524,25 @@
         <v>48</v>
       </c>
       <c r="B51" s="50" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C51" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D51" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="E51" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="E51" s="50" t="s">
+      <c r="F51" s="51" t="s">
         <v>192</v>
       </c>
-      <c r="F51" s="51" t="s">
+      <c r="G51" s="50" t="s">
         <v>193</v>
       </c>
-      <c r="G51" s="50" t="s">
-        <v>194</v>
-      </c>
       <c r="H51" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3552,25 +3551,25 @@
         <v>49</v>
       </c>
       <c r="B52" s="50" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C52" s="50" t="s">
         <v>28</v>
       </c>
       <c r="D52" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="E52" s="50" t="s">
         <v>110</v>
       </c>
-      <c r="E52" s="50" t="s">
+      <c r="F52" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="F52" s="51" t="s">
+      <c r="G52" s="50" t="s">
         <v>112</v>
       </c>
-      <c r="G52" s="50" t="s">
-        <v>113</v>
-      </c>
       <c r="H52" s="50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3732,172 +3731,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
-      <c r="N1" s="65"/>
-      <c r="O1" s="65"/>
-      <c r="P1" s="65"/>
-      <c r="Q1" s="65"/>
-      <c r="R1" s="65"/>
-      <c r="S1" s="65"/>
-      <c r="T1" s="65"/>
-      <c r="U1" s="65"/>
-      <c r="V1" s="65"/>
-      <c r="W1" s="65"/>
-      <c r="X1" s="65"/>
-      <c r="Y1" s="65"/>
-      <c r="Z1" s="65"/>
-      <c r="AA1" s="65"/>
-      <c r="AB1" s="65"/>
-      <c r="AC1" s="65"/>
-      <c r="AD1" s="65"/>
-      <c r="AE1" s="65"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
+      <c r="AE1" s="67"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="66" t="s">
+      <c r="C2" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="83" t="s">
+      <c r="D2" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="68" t="s">
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="77" t="s">
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="71"/>
+      <c r="Q2" s="72"/>
+      <c r="R2" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="78"/>
-      <c r="T2" s="78"/>
-      <c r="U2" s="78"/>
-      <c r="V2" s="78"/>
-      <c r="W2" s="78"/>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="78"/>
-      <c r="Z2" s="79"/>
-      <c r="AA2" s="58" t="s">
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="80"/>
+      <c r="V2" s="80"/>
+      <c r="W2" s="80"/>
+      <c r="X2" s="80"/>
+      <c r="Y2" s="80"/>
+      <c r="Z2" s="81"/>
+      <c r="AA2" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="59"/>
-      <c r="AC2" s="59"/>
-      <c r="AD2" s="59"/>
-      <c r="AE2" s="60"/>
+      <c r="AB2" s="61"/>
+      <c r="AC2" s="61"/>
+      <c r="AD2" s="61"/>
+      <c r="AE2" s="62"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="67"/>
-      <c r="B3" s="91"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="86" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="87"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="71" t="s">
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="72"/>
-      <c r="K3" s="72"/>
-      <c r="L3" s="72"/>
-      <c r="M3" s="72"/>
-      <c r="N3" s="72"/>
-      <c r="O3" s="72"/>
-      <c r="P3" s="72"/>
-      <c r="Q3" s="73"/>
-      <c r="R3" s="80" t="s">
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="74"/>
+      <c r="Q3" s="75"/>
+      <c r="R3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="81"/>
-      <c r="T3" s="81"/>
-      <c r="U3" s="81"/>
-      <c r="V3" s="81"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="81"/>
-      <c r="Y3" s="81"/>
-      <c r="Z3" s="82"/>
-      <c r="AA3" s="61" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="62"/>
-      <c r="AC3" s="62"/>
-      <c r="AD3" s="62"/>
-      <c r="AE3" s="63"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="83"/>
+      <c r="Z3" s="84"/>
+      <c r="AA3" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="65"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="67"/>
-      <c r="B4" s="91"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="89" t="s">
+      <c r="A4" s="69"/>
+      <c r="B4" s="93"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="91" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="76"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="78"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="74" t="s">
+      <c r="I4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="75"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="75"/>
-      <c r="M4" s="75"/>
-      <c r="N4" s="75"/>
-      <c r="O4" s="75"/>
-      <c r="P4" s="76"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="N4" s="77"/>
+      <c r="O4" s="77"/>
+      <c r="P4" s="78"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="74" t="s">
+      <c r="R4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="75"/>
-      <c r="T4" s="75"/>
-      <c r="U4" s="75"/>
-      <c r="V4" s="75"/>
-      <c r="W4" s="75"/>
-      <c r="X4" s="75"/>
-      <c r="Y4" s="76"/>
+      <c r="S4" s="77"/>
+      <c r="T4" s="77"/>
+      <c r="U4" s="77"/>
+      <c r="V4" s="77"/>
+      <c r="W4" s="77"/>
+      <c r="X4" s="77"/>
+      <c r="Y4" s="78"/>
       <c r="Z4" s="13"/>
-      <c r="AA4" s="64" t="s">
+      <c r="AA4" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="AB4" s="64"/>
-      <c r="AC4" s="64"/>
-      <c r="AD4" s="64"/>
+      <c r="AB4" s="66"/>
+      <c r="AC4" s="66"/>
+      <c r="AD4" s="66"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="67"/>
-      <c r="B5" s="91"/>
-      <c r="C5" s="67"/>
+      <c r="A5" s="69"/>
+      <c r="B5" s="93"/>
+      <c r="C5" s="69"/>
       <c r="D5" s="34"/>
       <c r="E5" s="34"/>
       <c r="F5" s="34"/>
@@ -7111,123 +7110,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="92"/>
-      <c r="T1" s="92"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="66" t="s">
+      <c r="C2" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="120" t="str">
+      <c r="D2" s="94" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="121"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="120" t="str">
+      <c r="E2" s="95"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="94" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="121"/>
-      <c r="I2" s="121"/>
-      <c r="J2" s="121"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="120" t="s">
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="121"/>
-      <c r="N2" s="121"/>
-      <c r="O2" s="121"/>
-      <c r="P2" s="122"/>
-      <c r="Q2" s="120" t="str">
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="96"/>
+      <c r="Q2" s="94" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="121"/>
-      <c r="S2" s="121"/>
-      <c r="T2" s="122"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="95"/>
+      <c r="T2" s="96"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="130"/>
-      <c r="B3" s="91"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="137" t="s">
+      <c r="A3" s="107"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="138"/>
-      <c r="F3" s="139"/>
-      <c r="G3" s="131" t="s">
+      <c r="E3" s="115"/>
+      <c r="F3" s="116"/>
+      <c r="G3" s="108" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="132"/>
-      <c r="I3" s="132"/>
-      <c r="J3" s="132"/>
-      <c r="K3" s="133"/>
-      <c r="L3" s="114" t="s">
+      <c r="H3" s="109"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="109"/>
+      <c r="K3" s="110"/>
+      <c r="L3" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="115"/>
-      <c r="N3" s="115"/>
-      <c r="O3" s="115"/>
-      <c r="P3" s="116"/>
-      <c r="Q3" s="123" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="124"/>
-      <c r="S3" s="124"/>
-      <c r="T3" s="125"/>
+      <c r="M3" s="140"/>
+      <c r="N3" s="140"/>
+      <c r="O3" s="140"/>
+      <c r="P3" s="141"/>
+      <c r="Q3" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="98"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="99"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="130"/>
-      <c r="B4" s="91"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="140"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="142"/>
-      <c r="G4" s="134"/>
-      <c r="H4" s="135"/>
-      <c r="I4" s="135"/>
-      <c r="J4" s="135"/>
-      <c r="K4" s="136"/>
-      <c r="L4" s="117"/>
-      <c r="M4" s="118"/>
-      <c r="N4" s="118"/>
-      <c r="O4" s="118"/>
-      <c r="P4" s="119"/>
-      <c r="Q4" s="126"/>
-      <c r="R4" s="127"/>
-      <c r="S4" s="127"/>
-      <c r="T4" s="128"/>
+      <c r="A4" s="107"/>
+      <c r="B4" s="93"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="117"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="112"/>
+      <c r="I4" s="112"/>
+      <c r="J4" s="112"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="142"/>
+      <c r="M4" s="143"/>
+      <c r="N4" s="143"/>
+      <c r="O4" s="143"/>
+      <c r="P4" s="144"/>
+      <c r="Q4" s="100"/>
+      <c r="R4" s="101"/>
+      <c r="S4" s="101"/>
+      <c r="T4" s="102"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="130"/>
-      <c r="B5" s="91"/>
-      <c r="C5" s="67"/>
+      <c r="A5" s="107"/>
+      <c r="B5" s="93"/>
+      <c r="C5" s="69"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9759,192 +9758,183 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="96" t="s">
+      <c r="D65" s="124" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="99" t="s">
+      <c r="E65" s="127" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="93" t="s">
+      <c r="G65" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="108" t="s">
+      <c r="H65" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="108" t="s">
+      <c r="I65" s="133" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="93" t="s">
+      <c r="J65" s="121" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="102" t="s">
+      <c r="L65" s="103" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="105" t="s">
+      <c r="M65" s="130" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="105" t="s">
+      <c r="N65" s="130" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="102" t="s">
+      <c r="O65" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="111" t="s">
+      <c r="Q65" s="136" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="111" t="s">
+      <c r="R65" s="136" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="111" t="s">
+      <c r="S65" s="136" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="97"/>
-      <c r="E66" s="100"/>
-      <c r="G66" s="94"/>
-      <c r="H66" s="109"/>
-      <c r="I66" s="109"/>
-      <c r="J66" s="94"/>
-      <c r="L66" s="103"/>
-      <c r="M66" s="106"/>
-      <c r="N66" s="106"/>
-      <c r="O66" s="103"/>
-      <c r="Q66" s="112"/>
-      <c r="R66" s="112"/>
-      <c r="S66" s="112"/>
+      <c r="D66" s="125"/>
+      <c r="E66" s="128"/>
+      <c r="G66" s="122"/>
+      <c r="H66" s="134"/>
+      <c r="I66" s="134"/>
+      <c r="J66" s="122"/>
+      <c r="L66" s="104"/>
+      <c r="M66" s="131"/>
+      <c r="N66" s="131"/>
+      <c r="O66" s="104"/>
+      <c r="Q66" s="137"/>
+      <c r="R66" s="137"/>
+      <c r="S66" s="137"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="97"/>
-      <c r="E67" s="100"/>
-      <c r="G67" s="94"/>
-      <c r="H67" s="109"/>
-      <c r="I67" s="109"/>
-      <c r="J67" s="94"/>
-      <c r="L67" s="103"/>
-      <c r="M67" s="106"/>
-      <c r="N67" s="106"/>
-      <c r="O67" s="103"/>
-      <c r="Q67" s="112"/>
-      <c r="R67" s="112"/>
-      <c r="S67" s="112"/>
+      <c r="D67" s="125"/>
+      <c r="E67" s="128"/>
+      <c r="G67" s="122"/>
+      <c r="H67" s="134"/>
+      <c r="I67" s="134"/>
+      <c r="J67" s="122"/>
+      <c r="L67" s="104"/>
+      <c r="M67" s="131"/>
+      <c r="N67" s="131"/>
+      <c r="O67" s="104"/>
+      <c r="Q67" s="137"/>
+      <c r="R67" s="137"/>
+      <c r="S67" s="137"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="97"/>
-      <c r="E68" s="100"/>
-      <c r="G68" s="94"/>
-      <c r="H68" s="109"/>
-      <c r="I68" s="109"/>
-      <c r="J68" s="94"/>
-      <c r="L68" s="103"/>
-      <c r="M68" s="106"/>
-      <c r="N68" s="106"/>
-      <c r="O68" s="103"/>
-      <c r="Q68" s="112"/>
-      <c r="R68" s="112"/>
-      <c r="S68" s="112"/>
+      <c r="D68" s="125"/>
+      <c r="E68" s="128"/>
+      <c r="G68" s="122"/>
+      <c r="H68" s="134"/>
+      <c r="I68" s="134"/>
+      <c r="J68" s="122"/>
+      <c r="L68" s="104"/>
+      <c r="M68" s="131"/>
+      <c r="N68" s="131"/>
+      <c r="O68" s="104"/>
+      <c r="Q68" s="137"/>
+      <c r="R68" s="137"/>
+      <c r="S68" s="137"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="97"/>
-      <c r="E69" s="100"/>
-      <c r="G69" s="94"/>
-      <c r="H69" s="109"/>
-      <c r="I69" s="109"/>
-      <c r="J69" s="94"/>
-      <c r="L69" s="103"/>
-      <c r="M69" s="106"/>
-      <c r="N69" s="106"/>
-      <c r="O69" s="103"/>
-      <c r="Q69" s="112"/>
-      <c r="R69" s="112"/>
-      <c r="S69" s="112"/>
+      <c r="D69" s="125"/>
+      <c r="E69" s="128"/>
+      <c r="G69" s="122"/>
+      <c r="H69" s="134"/>
+      <c r="I69" s="134"/>
+      <c r="J69" s="122"/>
+      <c r="L69" s="104"/>
+      <c r="M69" s="131"/>
+      <c r="N69" s="131"/>
+      <c r="O69" s="104"/>
+      <c r="Q69" s="137"/>
+      <c r="R69" s="137"/>
+      <c r="S69" s="137"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="97"/>
-      <c r="E70" s="100"/>
-      <c r="G70" s="94"/>
-      <c r="H70" s="109"/>
-      <c r="I70" s="109"/>
-      <c r="J70" s="94"/>
-      <c r="L70" s="103"/>
-      <c r="M70" s="106"/>
-      <c r="N70" s="106"/>
-      <c r="O70" s="103"/>
-      <c r="Q70" s="112"/>
-      <c r="R70" s="112"/>
-      <c r="S70" s="112"/>
+      <c r="D70" s="125"/>
+      <c r="E70" s="128"/>
+      <c r="G70" s="122"/>
+      <c r="H70" s="134"/>
+      <c r="I70" s="134"/>
+      <c r="J70" s="122"/>
+      <c r="L70" s="104"/>
+      <c r="M70" s="131"/>
+      <c r="N70" s="131"/>
+      <c r="O70" s="104"/>
+      <c r="Q70" s="137"/>
+      <c r="R70" s="137"/>
+      <c r="S70" s="137"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="97"/>
-      <c r="E71" s="100"/>
-      <c r="G71" s="94"/>
-      <c r="H71" s="109"/>
-      <c r="I71" s="109"/>
-      <c r="J71" s="94"/>
-      <c r="L71" s="103"/>
-      <c r="M71" s="106"/>
-      <c r="N71" s="106"/>
-      <c r="O71" s="103"/>
-      <c r="Q71" s="112"/>
-      <c r="R71" s="112"/>
-      <c r="S71" s="112"/>
+      <c r="D71" s="125"/>
+      <c r="E71" s="128"/>
+      <c r="G71" s="122"/>
+      <c r="H71" s="134"/>
+      <c r="I71" s="134"/>
+      <c r="J71" s="122"/>
+      <c r="L71" s="104"/>
+      <c r="M71" s="131"/>
+      <c r="N71" s="131"/>
+      <c r="O71" s="104"/>
+      <c r="Q71" s="137"/>
+      <c r="R71" s="137"/>
+      <c r="S71" s="137"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="97"/>
-      <c r="E72" s="100"/>
-      <c r="G72" s="94"/>
-      <c r="H72" s="109"/>
-      <c r="I72" s="109"/>
-      <c r="J72" s="94"/>
-      <c r="L72" s="103"/>
-      <c r="M72" s="106"/>
-      <c r="N72" s="106"/>
-      <c r="O72" s="103"/>
-      <c r="Q72" s="112"/>
-      <c r="R72" s="112"/>
-      <c r="S72" s="112"/>
+      <c r="D72" s="125"/>
+      <c r="E72" s="128"/>
+      <c r="G72" s="122"/>
+      <c r="H72" s="134"/>
+      <c r="I72" s="134"/>
+      <c r="J72" s="122"/>
+      <c r="L72" s="104"/>
+      <c r="M72" s="131"/>
+      <c r="N72" s="131"/>
+      <c r="O72" s="104"/>
+      <c r="Q72" s="137"/>
+      <c r="R72" s="137"/>
+      <c r="S72" s="137"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="97"/>
-      <c r="E73" s="100"/>
-      <c r="G73" s="94"/>
-      <c r="H73" s="109"/>
-      <c r="I73" s="109"/>
-      <c r="J73" s="94"/>
-      <c r="L73" s="103"/>
-      <c r="M73" s="106"/>
-      <c r="N73" s="106"/>
-      <c r="O73" s="103"/>
-      <c r="Q73" s="112"/>
-      <c r="R73" s="112"/>
-      <c r="S73" s="112"/>
+      <c r="D73" s="125"/>
+      <c r="E73" s="128"/>
+      <c r="G73" s="122"/>
+      <c r="H73" s="134"/>
+      <c r="I73" s="134"/>
+      <c r="J73" s="122"/>
+      <c r="L73" s="104"/>
+      <c r="M73" s="131"/>
+      <c r="N73" s="131"/>
+      <c r="O73" s="104"/>
+      <c r="Q73" s="137"/>
+      <c r="R73" s="137"/>
+      <c r="S73" s="137"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="98"/>
-      <c r="E74" s="101"/>
-      <c r="G74" s="95"/>
-      <c r="H74" s="110"/>
-      <c r="I74" s="110"/>
-      <c r="J74" s="95"/>
-      <c r="L74" s="104"/>
-      <c r="M74" s="107"/>
-      <c r="N74" s="107"/>
-      <c r="O74" s="104"/>
-      <c r="Q74" s="113"/>
-      <c r="R74" s="113"/>
-      <c r="S74" s="113"/>
+      <c r="D74" s="126"/>
+      <c r="E74" s="129"/>
+      <c r="G74" s="123"/>
+      <c r="H74" s="135"/>
+      <c r="I74" s="135"/>
+      <c r="J74" s="123"/>
+      <c r="L74" s="105"/>
+      <c r="M74" s="132"/>
+      <c r="N74" s="132"/>
+      <c r="O74" s="105"/>
+      <c r="Q74" s="138"/>
+      <c r="R74" s="138"/>
+      <c r="S74" s="138"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9961,6 +9951,15 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>